<commit_message>
fully cleaned GA ALNS
</commit_message>
<xml_diff>
--- a/hybrid_ph_mh_alns_seed_results.xlsx
+++ b/hybrid_ph_mh_alns_seed_results.xlsx
@@ -451,7 +451,7 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
@@ -589,7 +589,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.215</v>
+        <v>0.257</v>
       </c>
       <c r="J2" t="n">
         <v>20</v>
@@ -626,10 +626,10 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.839</v>
+        <v>0.965</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.623</v>
+        <v>0.708</v>
       </c>
       <c r="R2" t="n">
         <v>500</v>
@@ -684,7 +684,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.275</v>
+        <v>0.345</v>
       </c>
       <c r="J3" t="n">
         <v>20</v>
@@ -709,10 +709,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>1.578</v>
+        <v>2.029</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.302</v>
+        <v>1.683</v>
       </c>
       <c r="R3" t="n">
         <v>500</v>
@@ -755,7 +755,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -767,7 +767,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.289</v>
+        <v>0.335</v>
       </c>
       <c r="J4" t="n">
         <v>20</v>
@@ -792,10 +792,10 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>2.08</v>
+        <v>2.681</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.791</v>
+        <v>2.345</v>
       </c>
       <c r="R4" t="n">
         <v>500</v>
@@ -838,7 +838,7 @@
         <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F5" t="n">
         <v>11.1</v>
@@ -850,7 +850,7 @@
         <v>10</v>
       </c>
       <c r="I5" t="n">
-        <v>1.198</v>
+        <v>1.613</v>
       </c>
       <c r="J5" t="n">
         <v>38</v>
@@ -875,10 +875,10 @@
         <v>9</v>
       </c>
       <c r="P5" t="n">
-        <v>22.485</v>
+        <v>32.834</v>
       </c>
       <c r="Q5" t="n">
-        <v>21.286</v>
+        <v>31.219</v>
       </c>
       <c r="R5" t="n">
         <v>920.5</v>
@@ -921,7 +921,7 @@
         <v>28</v>
       </c>
       <c r="E6" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F6" t="n">
         <v>23.4</v>
@@ -933,7 +933,7 @@
         <v>22</v>
       </c>
       <c r="I6" t="n">
-        <v>3.285</v>
+        <v>2.95</v>
       </c>
       <c r="J6" t="n">
         <v>61</v>
@@ -958,10 +958,10 @@
         <v>19</v>
       </c>
       <c r="P6" t="n">
-        <v>68.23099999999999</v>
+        <v>67.09099999999999</v>
       </c>
       <c r="Q6" t="n">
-        <v>64.94499999999999</v>
+        <v>64.14</v>
       </c>
       <c r="R6" t="n">
         <v>829.7</v>
@@ -1004,7 +1004,7 @@
         <v>49</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="F7" t="n">
         <v>39.5</v>
@@ -1016,7 +1016,7 @@
         <v>36</v>
       </c>
       <c r="I7" t="n">
-        <v>5.506</v>
+        <v>5.796</v>
       </c>
       <c r="J7" t="n">
         <v>68.8</v>
@@ -1041,10 +1041,10 @@
         <v>32</v>
       </c>
       <c r="P7" t="n">
-        <v>158.33</v>
+        <v>213.183</v>
       </c>
       <c r="Q7" t="n">
-        <v>152.822</v>
+        <v>207.384</v>
       </c>
       <c r="R7" t="n">
         <v>959.5</v>
@@ -1099,7 +1099,7 @@
         <v>42</v>
       </c>
       <c r="I8" t="n">
-        <v>6.415</v>
+        <v>7.434</v>
       </c>
       <c r="J8" t="n">
         <v>91.2</v>
@@ -1124,17 +1124,17 @@
         <v>37</v>
       </c>
       <c r="P8" t="n">
-        <v>274.367</v>
+        <v>306.214</v>
       </c>
       <c r="Q8" t="n">
-        <v>267.95</v>
+        <v>298.779</v>
       </c>
       <c r="R8" t="n">
-        <v>1395.9</v>
+        <v>1364.9</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>it_lim,no_imp_lim</t>
+          <t>it_lim,no_imp_lim,t_lim</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1349,7 +1349,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.000347137451171875</v>
+        <v>0.0008101463317871094</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1361,7 +1361,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2137386798858643</v>
+        <v>0.2436573505401611</v>
       </c>
       <c r="K2" t="n">
         <v>20</v>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0.624800443649292</v>
+        <v>0.7148253917694092</v>
       </c>
       <c r="U2" t="n">
-        <v>0.8388862609863281</v>
+        <v>0.9592928886413574</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -1437,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0006144046783447266</v>
+        <v>0.0001778602600097656</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1449,7 +1449,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2000942230224609</v>
+        <v>0.2513082027435303</v>
       </c>
       <c r="K3" t="n">
         <v>20</v>
@@ -1481,10 +1481,10 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0.7156004905700684</v>
+        <v>0.7130506038665771</v>
       </c>
       <c r="U3" t="n">
-        <v>0.916309118270874</v>
+        <v>0.9645366668701172</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0003736019134521484</v>
+        <v>0.0003504753112792969</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2170369625091553</v>
+        <v>0.2757492065429688</v>
       </c>
       <c r="K4" t="n">
         <v>20</v>
@@ -1569,10 +1569,10 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.6380014419555664</v>
+        <v>0.6269407272338867</v>
       </c>
       <c r="U4" t="n">
-        <v>0.8554120063781738</v>
+        <v>0.9030404090881348</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0005788803100585938</v>
+        <v>0.0006835460662841797</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1625,7 +1625,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2206318378448486</v>
+        <v>0.2402288913726807</v>
       </c>
       <c r="K5" t="n">
         <v>20</v>
@@ -1657,10 +1657,10 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>0.6063680648803711</v>
+        <v>0.6857600212097168</v>
       </c>
       <c r="U5" t="n">
-        <v>0.8275787830352783</v>
+        <v>0.9266724586486816</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0006701946258544922</v>
+        <v>0.0002927780151367188</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1713,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2296895980834961</v>
+        <v>0.2570042610168457</v>
       </c>
       <c r="K6" t="n">
         <v>20</v>
@@ -1745,10 +1745,10 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0.6124095916748047</v>
+        <v>0.6889545917510986</v>
       </c>
       <c r="U6" t="n">
-        <v>0.8427693843841553</v>
+        <v>0.9462516307830811</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0008652210235595703</v>
+        <v>0.0002131462097167969</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1801,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2211434841156006</v>
+        <v>0.345083475112915</v>
       </c>
       <c r="K7" t="n">
         <v>20</v>
@@ -1833,10 +1833,10 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>0.6643798351287842</v>
+        <v>0.7694838047027588</v>
       </c>
       <c r="U7" t="n">
-        <v>0.8863885402679443</v>
+        <v>1.114780426025391</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -1877,7 +1877,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0006430149078369141</v>
+        <v>0.0006978511810302734</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1889,7 +1889,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2081694602966309</v>
+        <v>0.2448456287384033</v>
       </c>
       <c r="K8" t="n">
         <v>20</v>
@@ -1921,10 +1921,10 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.5690939426422119</v>
+        <v>0.6996982097625732</v>
       </c>
       <c r="U8" t="n">
-        <v>0.7779064178466797</v>
+        <v>0.9452416896820068</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003936290740966797</v>
+        <v>0.0005133152008056641</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.211479663848877</v>
+        <v>0.2346971035003662</v>
       </c>
       <c r="K9" t="n">
         <v>20</v>
@@ -2009,10 +2009,10 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0.5931298732757568</v>
+        <v>0.6943035125732422</v>
       </c>
       <c r="U9" t="n">
-        <v>0.8050031661987305</v>
+        <v>0.9295139312744141</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0008513927459716797</v>
+        <v>0.0001513957977294922</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -2065,7 +2065,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2134027481079102</v>
+        <v>0.2202522754669189</v>
       </c>
       <c r="K10" t="n">
         <v>20</v>
@@ -2097,10 +2097,10 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.6410448551177979</v>
+        <v>0.7941954135894775</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8552989959716797</v>
+        <v>1.014599084854126</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -2141,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0002954006195068359</v>
+        <v>0.0002985000610351562</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -2153,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2163703441619873</v>
+        <v>0.2533884048461914</v>
       </c>
       <c r="K11" t="n">
         <v>20</v>
@@ -2185,10 +2185,10 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.5688900947570801</v>
+        <v>0.6948974132537842</v>
       </c>
       <c r="U11" t="n">
-        <v>0.7855558395385742</v>
+        <v>0.9485843181610107</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
@@ -2229,7 +2229,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0006451606750488281</v>
+        <v>0.0004799365997314453</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -2241,7 +2241,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.2788460254669189</v>
+        <v>0.2699816226959229</v>
       </c>
       <c r="K12" t="n">
         <v>20</v>
@@ -2273,10 +2273,10 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>1.209953308105469</v>
+        <v>1.68302845954895</v>
       </c>
       <c r="U12" t="n">
-        <v>1.489444494247437</v>
+        <v>1.953490018844604</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0003719329833984375</v>
+        <v>0.0006096363067626953</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2581946849822998</v>
+        <v>0.2899844646453857</v>
       </c>
       <c r="K13" t="n">
         <v>20</v>
@@ -2361,10 +2361,10 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>1.324868679046631</v>
+        <v>1.700077772140503</v>
       </c>
       <c r="U13" t="n">
-        <v>1.583435297012329</v>
+        <v>1.990671873092651</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
@@ -2405,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0008485317230224609</v>
+        <v>0.0004365444183349609</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2691407203674316</v>
+        <v>0.3417923450469971</v>
       </c>
       <c r="K14" t="n">
         <v>20</v>
@@ -2449,10 +2449,10 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>1.286658763885498</v>
+        <v>1.64783501625061</v>
       </c>
       <c r="U14" t="n">
-        <v>1.556648015975952</v>
+        <v>1.990063905715942</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
@@ -2493,7 +2493,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0006935596466064453</v>
+        <v>0.0003387928009033203</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0.352391242980957</v>
+        <v>0.5219869613647461</v>
       </c>
       <c r="K15" t="n">
         <v>20</v>
@@ -2537,10 +2537,10 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>1.337256908416748</v>
+        <v>1.850628614425659</v>
       </c>
       <c r="U15" t="n">
-        <v>1.690341711044312</v>
+        <v>2.372954368591309</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.001165151596069336</v>
+        <v>0.0004634857177734375</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2593,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0.2761399745941162</v>
+        <v>0.2646429538726807</v>
       </c>
       <c r="K16" t="n">
         <v>20</v>
@@ -2625,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>1.41843581199646</v>
+        <v>1.726575374603271</v>
       </c>
       <c r="U16" t="n">
-        <v>1.695740938186646</v>
+        <v>1.991681814193726</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
@@ -2669,7 +2669,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0004184246063232422</v>
+        <v>0.0006275177001953125</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -2681,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.2691609859466553</v>
+        <v>0.3110785484313965</v>
       </c>
       <c r="K17" t="n">
         <v>20</v>
@@ -2713,10 +2713,10 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>1.210504293441772</v>
+        <v>1.499370813369751</v>
       </c>
       <c r="U17" t="n">
-        <v>1.480083703994751</v>
+        <v>1.811076879501343</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0004563331604003906</v>
+        <v>0.0005395412445068359</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -2769,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2528131008148193</v>
+        <v>0.3538327217102051</v>
       </c>
       <c r="K18" t="n">
         <v>20</v>
@@ -2801,10 +2801,10 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>1.407422780990601</v>
+        <v>1.85375452041626</v>
       </c>
       <c r="U18" t="n">
-        <v>1.66069221496582</v>
+        <v>2.208126783370972</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -2845,7 +2845,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0007131099700927734</v>
+        <v>0.0007336139678955078</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2857,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2725057601928711</v>
+        <v>0.3858168125152588</v>
       </c>
       <c r="K19" t="n">
         <v>20</v>
@@ -2889,10 +2889,10 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>1.268229246139526</v>
+        <v>1.614604949951172</v>
       </c>
       <c r="U19" t="n">
-        <v>1.54144811630249</v>
+        <v>2.001155376434326</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -2933,7 +2933,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0008614063262939453</v>
+        <v>0.0004825592041015625</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.2726516723632812</v>
+        <v>0.3656749725341797</v>
       </c>
       <c r="K20" t="n">
         <v>20</v>
@@ -2977,10 +2977,10 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>1.291438102722168</v>
+        <v>1.630741834640503</v>
       </c>
       <c r="U20" t="n">
-        <v>1.564951181411743</v>
+        <v>1.996899366378784</v>
       </c>
       <c r="V20" t="inlineStr">
         <is>
@@ -3021,7 +3021,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0006773471832275391</v>
+        <v>0.0006992816925048828</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -3033,7 +3033,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.2523255348205566</v>
+        <v>0.3480560779571533</v>
       </c>
       <c r="K21" t="n">
         <v>20</v>
@@ -3065,10 +3065,10 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>1.265780925750732</v>
+        <v>1.623961448669434</v>
       </c>
       <c r="U21" t="n">
-        <v>1.518783807754517</v>
+        <v>1.972716808319092</v>
       </c>
       <c r="V21" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0007104873657226562</v>
+        <v>0.0006122589111328125</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -3121,7 +3121,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0.2837071418762207</v>
+        <v>0.3497610092163086</v>
       </c>
       <c r="K22" t="n">
         <v>20</v>
@@ -3153,10 +3153,10 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>1.659703016281128</v>
+        <v>2.192342281341553</v>
       </c>
       <c r="U22" t="n">
-        <v>1.944120645523071</v>
+        <v>2.542715549468994</v>
       </c>
       <c r="V22" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0004227161407470703</v>
+        <v>0.0005695819854736328</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -3209,7 +3209,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0.2899181842803955</v>
+        <v>0.3599486351013184</v>
       </c>
       <c r="K23" t="n">
         <v>20</v>
@@ -3241,10 +3241,10 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>1.783647060394287</v>
+        <v>2.517016887664795</v>
       </c>
       <c r="U23" t="n">
-        <v>2.07398796081543</v>
+        <v>2.877535104751587</v>
       </c>
       <c r="V23" t="inlineStr">
         <is>
@@ -3285,7 +3285,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0008208751678466797</v>
+        <v>0.0005385875701904297</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.3045756816864014</v>
+        <v>0.2947931289672852</v>
       </c>
       <c r="K24" t="n">
         <v>20</v>
@@ -3329,10 +3329,10 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>1.891098022460938</v>
+        <v>2.445166349411011</v>
       </c>
       <c r="U24" t="n">
-        <v>2.196494579315186</v>
+        <v>2.740498065948486</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0.000453948974609375</v>
+        <v>0.0005786418914794922</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -3385,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0.2984228134155273</v>
+        <v>0.3339593410491943</v>
       </c>
       <c r="K25" t="n">
         <v>20</v>
@@ -3417,10 +3417,10 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>1.691244602203369</v>
+        <v>2.265771865844727</v>
       </c>
       <c r="U25" t="n">
-        <v>1.990121364593506</v>
+        <v>2.6003098487854</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0005567073822021484</v>
+        <v>0.0003895759582519531</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -3473,7 +3473,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0.2756173610687256</v>
+        <v>0.4103050231933594</v>
       </c>
       <c r="K26" t="n">
         <v>20</v>
@@ -3505,10 +3505,10 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>1.777453184127808</v>
+        <v>2.335699319839478</v>
       </c>
       <c r="U26" t="n">
-        <v>2.053627252578735</v>
+        <v>2.746393918991089</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
@@ -3549,7 +3549,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0006210803985595703</v>
+        <v>0.0004220008850097656</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -3561,7 +3561,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0.2818522453308105</v>
+        <v>0.3233263492584229</v>
       </c>
       <c r="K27" t="n">
         <v>20</v>
@@ -3593,10 +3593,10 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>1.772819995880127</v>
+        <v>2.376081705093384</v>
       </c>
       <c r="U27" t="n">
-        <v>2.055293321609497</v>
+        <v>2.699830055236816</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
@@ -3637,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0008776187896728516</v>
+        <v>0.000476837158203125</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0.3061959743499756</v>
+        <v>0.3205084800720215</v>
       </c>
       <c r="K28" t="n">
         <v>20</v>
@@ -3681,10 +3681,10 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>1.916248798370361</v>
+        <v>2.512481689453125</v>
       </c>
       <c r="U28" t="n">
-        <v>2.22332239151001</v>
+        <v>2.83346700668335</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
@@ -3725,7 +3725,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0006625652313232422</v>
+        <v>0.0004911422729492188</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -3737,7 +3737,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0.266387939453125</v>
+        <v>0.3357155323028564</v>
       </c>
       <c r="K29" t="n">
         <v>20</v>
@@ -3769,10 +3769,10 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>1.743336200714111</v>
+        <v>2.144961833953857</v>
       </c>
       <c r="U29" t="n">
-        <v>2.01038670539856</v>
+        <v>2.481168508529663</v>
       </c>
       <c r="V29" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0008573532104492188</v>
+        <v>0.0004134178161621094</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -3825,7 +3825,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0.2936575412750244</v>
+        <v>0.314018726348877</v>
       </c>
       <c r="K30" t="n">
         <v>20</v>
@@ -3857,10 +3857,10 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>1.784942626953125</v>
+        <v>2.324721097946167</v>
       </c>
       <c r="U30" t="n">
-        <v>2.079457521438599</v>
+        <v>2.639153242111206</v>
       </c>
       <c r="V30" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0007123947143554688</v>
+        <v>0.0004088878631591797</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2876307964324951</v>
+        <v>0.3098609447479248</v>
       </c>
       <c r="K31" t="n">
         <v>20</v>
@@ -3945,10 +3945,10 @@
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>1.887743234634399</v>
+        <v>2.33649468421936</v>
       </c>
       <c r="U31" t="n">
-        <v>2.17608642578125</v>
+        <v>2.646764516830444</v>
       </c>
       <c r="V31" t="inlineStr">
         <is>
@@ -3989,7 +3989,7 @@
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>0.001035690307617188</v>
+        <v>0.001375675201416016</v>
       </c>
       <c r="G32" t="n">
         <v>12</v>
@@ -4001,7 +4001,7 @@
         <v>12</v>
       </c>
       <c r="J32" t="n">
-        <v>0.9648752212524414</v>
+        <v>1.170994520187378</v>
       </c>
       <c r="K32" t="n">
         <v>31</v>
@@ -4033,10 +4033,10 @@
         <v>9</v>
       </c>
       <c r="T32" t="n">
-        <v>26.69189119338989</v>
+        <v>39.22724962234497</v>
       </c>
       <c r="U32" t="n">
-        <v>27.65780210494995</v>
+        <v>40.39961981773376</v>
       </c>
       <c r="V32" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
         <v>16</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0008776187896728516</v>
+        <v>0.001531600952148438</v>
       </c>
       <c r="G33" t="n">
         <v>11</v>
@@ -4089,7 +4089,7 @@
         <v>11</v>
       </c>
       <c r="J33" t="n">
-        <v>0.9880061149597168</v>
+        <v>1.310221433639526</v>
       </c>
       <c r="K33" t="n">
         <v>33</v>
@@ -4121,10 +4121,10 @@
         <v>9</v>
       </c>
       <c r="T33" t="n">
-        <v>19.51586365699768</v>
+        <v>29.58467650413513</v>
       </c>
       <c r="U33" t="n">
-        <v>20.50474739074707</v>
+        <v>30.89642953872681</v>
       </c>
       <c r="V33" t="inlineStr">
         <is>
@@ -4165,7 +4165,7 @@
         <v>16</v>
       </c>
       <c r="F34" t="n">
-        <v>0.001096010208129883</v>
+        <v>0.0008275508880615234</v>
       </c>
       <c r="G34" t="n">
         <v>12</v>
@@ -4177,7 +4177,7 @@
         <v>12</v>
       </c>
       <c r="J34" t="n">
-        <v>1.040075778961182</v>
+        <v>1.440778493881226</v>
       </c>
       <c r="K34" t="n">
         <v>35</v>
@@ -4209,10 +4209,10 @@
         <v>10</v>
       </c>
       <c r="T34" t="n">
-        <v>16.07514715194702</v>
+        <v>24.61968851089478</v>
       </c>
       <c r="U34" t="n">
-        <v>17.11631894111633</v>
+        <v>26.06129455566406</v>
       </c>
       <c r="V34" t="inlineStr">
         <is>
@@ -4253,7 +4253,7 @@
         <v>14</v>
       </c>
       <c r="F35" t="n">
-        <v>0.001061201095581055</v>
+        <v>0.001179695129394531</v>
       </c>
       <c r="G35" t="n">
         <v>11</v>
@@ -4265,7 +4265,7 @@
         <v>11</v>
       </c>
       <c r="J35" t="n">
-        <v>1.03676176071167</v>
+        <v>1.447726249694824</v>
       </c>
       <c r="K35" t="n">
         <v>35</v>
@@ -4297,10 +4297,10 @@
         <v>9</v>
       </c>
       <c r="T35" t="n">
-        <v>13.54414629936218</v>
+        <v>19.97590231895447</v>
       </c>
       <c r="U35" t="n">
-        <v>14.58196926116943</v>
+        <v>21.42480826377869</v>
       </c>
       <c r="V35" t="inlineStr">
         <is>
@@ -4341,7 +4341,7 @@
         <v>16</v>
       </c>
       <c r="F36" t="n">
-        <v>0.001188278198242188</v>
+        <v>0.001357793807983398</v>
       </c>
       <c r="G36" t="n">
         <v>11</v>
@@ -4353,7 +4353,7 @@
         <v>11</v>
       </c>
       <c r="J36" t="n">
-        <v>1.747039318084717</v>
+        <v>2.52549409866333</v>
       </c>
       <c r="K36" t="n">
         <v>45</v>
@@ -4385,10 +4385,10 @@
         <v>9</v>
       </c>
       <c r="T36" t="n">
-        <v>21.19950008392334</v>
+        <v>30.57473802566528</v>
       </c>
       <c r="U36" t="n">
-        <v>22.9477276802063</v>
+        <v>33.1015899181366</v>
       </c>
       <c r="V36" t="inlineStr">
         <is>
@@ -4429,7 +4429,7 @@
         <v>14</v>
       </c>
       <c r="F37" t="n">
-        <v>0.0008656978607177734</v>
+        <v>0.001788616180419922</v>
       </c>
       <c r="G37" t="n">
         <v>11</v>
@@ -4441,7 +4441,7 @@
         <v>11</v>
       </c>
       <c r="J37" t="n">
-        <v>1.251269578933716</v>
+        <v>1.666623115539551</v>
       </c>
       <c r="K37" t="n">
         <v>41</v>
@@ -4473,10 +4473,10 @@
         <v>9</v>
       </c>
       <c r="T37" t="n">
-        <v>23.70487785339355</v>
+        <v>35.10482335090637</v>
       </c>
       <c r="U37" t="n">
-        <v>24.95701313018799</v>
+        <v>36.77323508262634</v>
       </c>
       <c r="V37" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>14</v>
       </c>
       <c r="F38" t="n">
-        <v>0.001590490341186523</v>
+        <v>0.001896381378173828</v>
       </c>
       <c r="G38" t="n">
         <v>10</v>
@@ -4529,7 +4529,7 @@
         <v>10</v>
       </c>
       <c r="J38" t="n">
-        <v>1.460759401321411</v>
+        <v>1.894102096557617</v>
       </c>
       <c r="K38" t="n">
         <v>45</v>
@@ -4561,10 +4561,10 @@
         <v>9</v>
       </c>
       <c r="T38" t="n">
-        <v>21.38955283164978</v>
+        <v>31.64168238639832</v>
       </c>
       <c r="U38" t="n">
-        <v>22.85190272331238</v>
+        <v>33.53768086433411</v>
       </c>
       <c r="V38" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         <v>16</v>
       </c>
       <c r="F39" t="n">
-        <v>0.001565217971801758</v>
+        <v>0.002011775970458984</v>
       </c>
       <c r="G39" t="n">
         <v>11</v>
@@ -4617,7 +4617,7 @@
         <v>11</v>
       </c>
       <c r="J39" t="n">
-        <v>1.386668920516968</v>
+        <v>1.734522819519043</v>
       </c>
       <c r="K39" t="n">
         <v>44</v>
@@ -4649,10 +4649,10 @@
         <v>9</v>
       </c>
       <c r="T39" t="n">
-        <v>17.1313488483429</v>
+        <v>25.88877987861633</v>
       </c>
       <c r="U39" t="n">
-        <v>18.51958298683167</v>
+        <v>27.62531447410583</v>
       </c>
       <c r="V39" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         <v>15</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0009636878967285156</v>
+        <v>0.001261472702026367</v>
       </c>
       <c r="G40" t="n">
         <v>11</v>
@@ -4705,7 +4705,7 @@
         <v>11</v>
       </c>
       <c r="J40" t="n">
-        <v>0.9980344772338867</v>
+        <v>1.367206573486328</v>
       </c>
       <c r="K40" t="n">
         <v>34</v>
@@ -4737,10 +4737,10 @@
         <v>9</v>
       </c>
       <c r="T40" t="n">
-        <v>28.320481300354</v>
+        <v>43.41889977455139</v>
       </c>
       <c r="U40" t="n">
-        <v>29.31947946548462</v>
+        <v>44.78736782073975</v>
       </c>
       <c r="V40" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
         <v>16</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0009126663208007812</v>
+        <v>0.002079248428344727</v>
       </c>
       <c r="G41" t="n">
         <v>11</v>
@@ -4793,7 +4793,7 @@
         <v>11</v>
       </c>
       <c r="J41" t="n">
-        <v>1.109433174133301</v>
+        <v>1.570752859115601</v>
       </c>
       <c r="K41" t="n">
         <v>37</v>
@@ -4825,10 +4825,10 @@
         <v>9</v>
       </c>
       <c r="T41" t="n">
-        <v>25.28454303741455</v>
+        <v>32.1569197177887</v>
       </c>
       <c r="U41" t="n">
-        <v>26.39488887786865</v>
+        <v>33.72975182533264</v>
       </c>
       <c r="V41" t="inlineStr">
         <is>
@@ -4869,7 +4869,7 @@
         <v>29</v>
       </c>
       <c r="F42" t="n">
-        <v>0.00106358528137207</v>
+        <v>0.0009019374847412109</v>
       </c>
       <c r="G42" t="n">
         <v>22</v>
@@ -4881,7 +4881,7 @@
         <v>22</v>
       </c>
       <c r="J42" t="n">
-        <v>3.793851137161255</v>
+        <v>3.464616060256958</v>
       </c>
       <c r="K42" t="n">
         <v>69</v>
@@ -4913,10 +4913,10 @@
         <v>20</v>
       </c>
       <c r="T42" t="n">
-        <v>55.13903141021729</v>
+        <v>56.31191802024841</v>
       </c>
       <c r="U42" t="n">
-        <v>58.93394613265991</v>
+        <v>59.77743601799011</v>
       </c>
       <c r="V42" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         <v>35</v>
       </c>
       <c r="F43" t="n">
-        <v>0.002321243286132812</v>
+        <v>0.001275777816772461</v>
       </c>
       <c r="G43" t="n">
         <v>23</v>
@@ -4969,7 +4969,7 @@
         <v>23</v>
       </c>
       <c r="J43" t="n">
-        <v>2.702383279800415</v>
+        <v>2.351820468902588</v>
       </c>
       <c r="K43" t="n">
         <v>59</v>
@@ -5001,10 +5001,10 @@
         <v>20</v>
       </c>
       <c r="T43" t="n">
-        <v>60.85281467437744</v>
+        <v>61.94121789932251</v>
       </c>
       <c r="U43" t="n">
-        <v>63.55751919746399</v>
+        <v>64.29431414604187</v>
       </c>
       <c r="V43" t="inlineStr">
         <is>
@@ -5045,7 +5045,7 @@
         <v>29</v>
       </c>
       <c r="F44" t="n">
-        <v>0.003142595291137695</v>
+        <v>0.001931428909301758</v>
       </c>
       <c r="G44" t="n">
         <v>24</v>
@@ -5057,7 +5057,7 @@
         <v>24</v>
       </c>
       <c r="J44" t="n">
-        <v>2.304579496383667</v>
+        <v>2.016704082489014</v>
       </c>
       <c r="K44" t="n">
         <v>51</v>
@@ -5089,10 +5089,10 @@
         <v>20</v>
       </c>
       <c r="T44" t="n">
-        <v>39.44452929496765</v>
+        <v>40.77013659477234</v>
       </c>
       <c r="U44" t="n">
-        <v>41.75225138664246</v>
+        <v>42.78877210617065</v>
       </c>
       <c r="V44" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
         <v>30</v>
       </c>
       <c r="F45" t="n">
-        <v>0.001340627670288086</v>
+        <v>0.00177764892578125</v>
       </c>
       <c r="G45" t="n">
         <v>22</v>
@@ -5145,7 +5145,7 @@
         <v>22</v>
       </c>
       <c r="J45" t="n">
-        <v>3.019871950149536</v>
+        <v>2.494786977767944</v>
       </c>
       <c r="K45" t="n">
         <v>62</v>
@@ -5177,10 +5177,10 @@
         <v>19</v>
       </c>
       <c r="T45" t="n">
-        <v>70.94095158576965</v>
+        <v>72.76348805427551</v>
       </c>
       <c r="U45" t="n">
-        <v>73.96216416358948</v>
+        <v>75.26005268096924</v>
       </c>
       <c r="V45" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         <v>34</v>
       </c>
       <c r="F46" t="n">
-        <v>0.001890659332275391</v>
+        <v>0.001365900039672852</v>
       </c>
       <c r="G46" t="n">
         <v>23</v>
@@ -5233,7 +5233,7 @@
         <v>23</v>
       </c>
       <c r="J46" t="n">
-        <v>3.437214374542236</v>
+        <v>3.412692308425903</v>
       </c>
       <c r="K46" t="n">
         <v>69</v>
@@ -5265,10 +5265,10 @@
         <v>20</v>
       </c>
       <c r="T46" t="n">
-        <v>63.33185529708862</v>
+        <v>48.28197240829468</v>
       </c>
       <c r="U46" t="n">
-        <v>66.77096033096313</v>
+        <v>51.69603061676025</v>
       </c>
       <c r="V46" t="inlineStr">
         <is>
@@ -5309,7 +5309,7 @@
         <v>30</v>
       </c>
       <c r="F47" t="n">
-        <v>0.00138401985168457</v>
+        <v>0.001113653182983398</v>
       </c>
       <c r="G47" t="n">
         <v>24</v>
@@ -5321,7 +5321,7 @@
         <v>24</v>
       </c>
       <c r="J47" t="n">
-        <v>2.442933797836304</v>
+        <v>1.672097444534302</v>
       </c>
       <c r="K47" t="n">
         <v>44</v>
@@ -5353,10 +5353,10 @@
         <v>20</v>
       </c>
       <c r="T47" t="n">
-        <v>72.22267270088196</v>
+        <v>66.96747064590454</v>
       </c>
       <c r="U47" t="n">
-        <v>74.66699051856995</v>
+        <v>68.64068174362183</v>
       </c>
       <c r="V47" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
         <v>32</v>
       </c>
       <c r="F48" t="n">
-        <v>0.001450777053833008</v>
+        <v>0.001384735107421875</v>
       </c>
       <c r="G48" t="n">
         <v>25</v>
@@ -5409,7 +5409,7 @@
         <v>25</v>
       </c>
       <c r="J48" t="n">
-        <v>5.235860109329224</v>
+        <v>3.474217176437378</v>
       </c>
       <c r="K48" t="n">
         <v>85</v>
@@ -5441,10 +5441,10 @@
         <v>19</v>
       </c>
       <c r="T48" t="n">
-        <v>91.30044651031494</v>
+        <v>76.89169049263</v>
       </c>
       <c r="U48" t="n">
-        <v>96.537757396698</v>
+        <v>80.3672924041748</v>
       </c>
       <c r="V48" t="inlineStr">
         <is>
@@ -5485,7 +5485,7 @@
         <v>33</v>
       </c>
       <c r="F49" t="n">
-        <v>0.002431154251098633</v>
+        <v>0.001802682876586914</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -5497,7 +5497,7 @@
         <v>26</v>
       </c>
       <c r="J49" t="n">
-        <v>2.594558477401733</v>
+        <v>1.898383378982544</v>
       </c>
       <c r="K49" t="n">
         <v>49</v>
@@ -5529,10 +5529,10 @@
         <v>20</v>
       </c>
       <c r="T49" t="n">
-        <v>78.05465722084045</v>
+        <v>78.91547346115112</v>
       </c>
       <c r="U49" t="n">
-        <v>80.65164685249329</v>
+        <v>80.81565952301025</v>
       </c>
       <c r="V49" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v>28</v>
       </c>
       <c r="F50" t="n">
-        <v>0.00130462646484375</v>
+        <v>0.001923084259033203</v>
       </c>
       <c r="G50" t="n">
         <v>23</v>
@@ -5585,7 +5585,7 @@
         <v>23</v>
       </c>
       <c r="J50" t="n">
-        <v>4.029046773910522</v>
+        <v>4.141350746154785</v>
       </c>
       <c r="K50" t="n">
         <v>65</v>
@@ -5617,10 +5617,10 @@
         <v>19</v>
       </c>
       <c r="T50" t="n">
-        <v>73.07584238052368</v>
+        <v>84.49457049369812</v>
       </c>
       <c r="U50" t="n">
-        <v>77.10619378089905</v>
+        <v>88.63784432411194</v>
       </c>
       <c r="V50" t="inlineStr">
         <is>
@@ -5661,7 +5661,7 @@
         <v>35</v>
       </c>
       <c r="F51" t="n">
-        <v>0.002309322357177734</v>
+        <v>0.001408815383911133</v>
       </c>
       <c r="G51" t="n">
         <v>22</v>
@@ -5673,7 +5673,7 @@
         <v>22</v>
       </c>
       <c r="J51" t="n">
-        <v>3.28545093536377</v>
+        <v>4.571100950241089</v>
       </c>
       <c r="K51" t="n">
         <v>57</v>
@@ -5705,10 +5705,10 @@
         <v>21</v>
       </c>
       <c r="T51" t="n">
-        <v>45.08503603935242</v>
+        <v>54.05926036834717</v>
       </c>
       <c r="U51" t="n">
-        <v>48.37279629707336</v>
+        <v>58.63177013397217</v>
       </c>
       <c r="V51" t="inlineStr">
         <is>
@@ -5749,7 +5749,7 @@
         <v>54</v>
       </c>
       <c r="F52" t="n">
-        <v>0.003355979919433594</v>
+        <v>0.001282691955566406</v>
       </c>
       <c r="G52" t="n">
         <v>36</v>
@@ -5761,7 +5761,7 @@
         <v>36</v>
       </c>
       <c r="J52" t="n">
-        <v>5.979092359542847</v>
+        <v>8.18970799446106</v>
       </c>
       <c r="K52" t="n">
         <v>74</v>
@@ -5793,10 +5793,10 @@
         <v>34</v>
       </c>
       <c r="T52" t="n">
-        <v>148.7658965587616</v>
+        <v>181.0873084068298</v>
       </c>
       <c r="U52" t="n">
-        <v>154.7483448982239</v>
+        <v>189.2782990932465</v>
       </c>
       <c r="V52" t="inlineStr">
         <is>
@@ -5837,7 +5837,7 @@
         <v>59</v>
       </c>
       <c r="F53" t="n">
-        <v>0.002090930938720703</v>
+        <v>0.001517534255981445</v>
       </c>
       <c r="G53" t="n">
         <v>40</v>
@@ -5849,7 +5849,7 @@
         <v>40</v>
       </c>
       <c r="J53" t="n">
-        <v>5.551863193511963</v>
+        <v>7.621034145355225</v>
       </c>
       <c r="K53" t="n">
         <v>75</v>
@@ -5881,10 +5881,10 @@
         <v>36</v>
       </c>
       <c r="T53" t="n">
-        <v>100.6322181224823</v>
+        <v>111.8289468288422</v>
       </c>
       <c r="U53" t="n">
-        <v>106.186172246933</v>
+        <v>119.4514985084534</v>
       </c>
       <c r="V53" t="inlineStr">
         <is>
@@ -5925,7 +5925,7 @@
         <v>54</v>
       </c>
       <c r="F54" t="n">
-        <v>0.002240896224975586</v>
+        <v>0.00830078125</v>
       </c>
       <c r="G54" t="n">
         <v>39</v>
@@ -5937,7 +5937,7 @@
         <v>39</v>
       </c>
       <c r="J54" t="n">
-        <v>4.224680662155151</v>
+        <v>6.503918647766113</v>
       </c>
       <c r="K54" t="n">
         <v>68</v>
@@ -5969,10 +5969,10 @@
         <v>32</v>
       </c>
       <c r="T54" t="n">
-        <v>226.8178315162659</v>
+        <v>201.4471638202667</v>
       </c>
       <c r="U54" t="n">
-        <v>231.044753074646</v>
+        <v>207.9593832492828</v>
       </c>
       <c r="V54" t="inlineStr">
         <is>
@@ -6013,7 +6013,7 @@
         <v>53</v>
       </c>
       <c r="F55" t="n">
-        <v>0.004796266555786133</v>
+        <v>0.002784013748168945</v>
       </c>
       <c r="G55" t="n">
         <v>42</v>
@@ -6025,7 +6025,7 @@
         <v>42</v>
       </c>
       <c r="J55" t="n">
-        <v>16.04381060600281</v>
+        <v>4.440566778182983</v>
       </c>
       <c r="K55" t="n">
         <v>69</v>
@@ -6057,10 +6057,10 @@
         <v>35</v>
       </c>
       <c r="T55" t="n">
-        <v>134.5764470100403</v>
+        <v>145.4961667060852</v>
       </c>
       <c r="U55" t="n">
-        <v>150.6250538825989</v>
+        <v>149.9395174980164</v>
       </c>
       <c r="V55" t="inlineStr">
         <is>
@@ -6101,7 +6101,7 @@
         <v>56</v>
       </c>
       <c r="F56" t="n">
-        <v>0.001654386520385742</v>
+        <v>0.001832246780395508</v>
       </c>
       <c r="G56" t="n">
         <v>39</v>
@@ -6113,7 +6113,7 @@
         <v>39</v>
       </c>
       <c r="J56" t="n">
-        <v>4.439785718917847</v>
+        <v>4.726808786392212</v>
       </c>
       <c r="K56" t="n">
         <v>69</v>
@@ -6145,10 +6145,10 @@
         <v>33</v>
       </c>
       <c r="T56" t="n">
-        <v>119.2966840267181</v>
+        <v>189.0848925113678</v>
       </c>
       <c r="U56" t="n">
-        <v>123.7381241321564</v>
+        <v>193.8135335445404</v>
       </c>
       <c r="V56" t="inlineStr">
         <is>
@@ -6189,7 +6189,7 @@
         <v>51</v>
       </c>
       <c r="F57" t="n">
-        <v>0.001036167144775391</v>
+        <v>0.001629114151000977</v>
       </c>
       <c r="G57" t="n">
         <v>42</v>
@@ -6201,7 +6201,7 @@
         <v>42</v>
       </c>
       <c r="J57" t="n">
-        <v>2.950500249862671</v>
+        <v>4.116897344589233</v>
       </c>
       <c r="K57" t="n">
         <v>58</v>
@@ -6233,10 +6233,10 @@
         <v>38</v>
       </c>
       <c r="T57" t="n">
-        <v>72.36353182792664</v>
+        <v>99.97208905220032</v>
       </c>
       <c r="U57" t="n">
-        <v>75.31506824493408</v>
+        <v>104.0906155109406</v>
       </c>
       <c r="V57" t="inlineStr">
         <is>
@@ -6277,7 +6277,7 @@
         <v>56</v>
       </c>
       <c r="F58" t="n">
-        <v>0.002232074737548828</v>
+        <v>0.001563072204589844</v>
       </c>
       <c r="G58" t="n">
         <v>39</v>
@@ -6289,7 +6289,7 @@
         <v>39</v>
       </c>
       <c r="J58" t="n">
-        <v>4.658681392669678</v>
+        <v>5.763643026351929</v>
       </c>
       <c r="K58" t="n">
         <v>74</v>
@@ -6321,10 +6321,10 @@
         <v>38</v>
       </c>
       <c r="T58" t="n">
-        <v>73.40750288963318</v>
+        <v>88.6357409954071</v>
       </c>
       <c r="U58" t="n">
-        <v>78.06841635704041</v>
+        <v>94.40094709396362</v>
       </c>
       <c r="V58" t="inlineStr">
         <is>
@@ -6365,7 +6365,7 @@
         <v>54</v>
       </c>
       <c r="F59" t="n">
-        <v>0.001161813735961914</v>
+        <v>0.002349138259887695</v>
       </c>
       <c r="G59" t="n">
         <v>41</v>
@@ -6377,7 +6377,7 @@
         <v>41</v>
       </c>
       <c r="J59" t="n">
-        <v>3.662752628326416</v>
+        <v>4.875472784042358</v>
       </c>
       <c r="K59" t="n">
         <v>70</v>
@@ -6409,10 +6409,10 @@
         <v>33</v>
       </c>
       <c r="T59" t="n">
-        <v>180.5149443149567</v>
+        <v>217.1243646144867</v>
       </c>
       <c r="U59" t="n">
-        <v>184.178858757019</v>
+        <v>222.0021865367889</v>
       </c>
       <c r="V59" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
         <v>49</v>
       </c>
       <c r="F60" t="n">
-        <v>0.001051664352416992</v>
+        <v>0.003035068511962891</v>
       </c>
       <c r="G60" t="n">
         <v>38</v>
@@ -6465,7 +6465,7 @@
         <v>38</v>
       </c>
       <c r="J60" t="n">
-        <v>3.645114898681641</v>
+        <v>5.305437326431274</v>
       </c>
       <c r="K60" t="n">
         <v>58</v>
@@ -6497,10 +6497,10 @@
         <v>33</v>
       </c>
       <c r="T60" t="n">
-        <v>270.9640567302704</v>
+        <v>346.1360051631927</v>
       </c>
       <c r="U60" t="n">
-        <v>274.6102232933044</v>
+        <v>351.444477558136</v>
       </c>
       <c r="V60" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         <v>55</v>
       </c>
       <c r="F61" t="n">
-        <v>0.001082897186279297</v>
+        <v>0.00164484977722168</v>
       </c>
       <c r="G61" t="n">
         <v>39</v>
@@ -6553,7 +6553,7 @@
         <v>39</v>
       </c>
       <c r="J61" t="n">
-        <v>3.906474351882935</v>
+        <v>6.417054414749146</v>
       </c>
       <c r="K61" t="n">
         <v>73</v>
@@ -6585,10 +6585,10 @@
         <v>34</v>
       </c>
       <c r="T61" t="n">
-        <v>200.8792588710785</v>
+        <v>493.0264613628387</v>
       </c>
       <c r="U61" t="n">
-        <v>204.7868161201477</v>
+        <v>499.4451606273651</v>
       </c>
       <c r="V61" t="inlineStr">
         <is>
@@ -6629,7 +6629,7 @@
         <v>59</v>
       </c>
       <c r="F62" t="n">
-        <v>0.00134587287902832</v>
+        <v>0.002321720123291016</v>
       </c>
       <c r="G62" t="n">
         <v>50</v>
@@ -6641,7 +6641,7 @@
         <v>50</v>
       </c>
       <c r="J62" t="n">
-        <v>4.072217702865601</v>
+        <v>5.665124416351318</v>
       </c>
       <c r="K62" t="n">
         <v>63</v>
@@ -6673,10 +6673,10 @@
         <v>39</v>
       </c>
       <c r="T62" t="n">
-        <v>342.6690044403076</v>
+        <v>600.4185683727264</v>
       </c>
       <c r="U62" t="n">
-        <v>346.7425680160522</v>
+        <v>606.086014509201</v>
       </c>
       <c r="V62" t="inlineStr">
         <is>
@@ -6687,11 +6687,11 @@
         <v>1</v>
       </c>
       <c r="X62" t="n">
-        <v>1608</v>
+        <v>1298</v>
       </c>
       <c r="Y62" t="inlineStr">
         <is>
-          <t>no_imp_lim</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="Z62" t="n">
@@ -6717,7 +6717,7 @@
         <v>65</v>
       </c>
       <c r="F63" t="n">
-        <v>0.001293659210205078</v>
+        <v>0.001754999160766602</v>
       </c>
       <c r="G63" t="n">
         <v>42</v>
@@ -6729,7 +6729,7 @@
         <v>42</v>
       </c>
       <c r="J63" t="n">
-        <v>8.99919867515564</v>
+        <v>8.501379013061523</v>
       </c>
       <c r="K63" t="n">
         <v>128</v>
@@ -6761,10 +6761,10 @@
         <v>39</v>
       </c>
       <c r="T63" t="n">
-        <v>270.610095500946</v>
+        <v>243.6602087020874</v>
       </c>
       <c r="U63" t="n">
-        <v>279.6105878353119</v>
+        <v>252.1633427143097</v>
       </c>
       <c r="V63" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>65</v>
       </c>
       <c r="F64" t="n">
-        <v>0.001281976699829102</v>
+        <v>0.001955270767211914</v>
       </c>
       <c r="G64" t="n">
         <v>47</v>
@@ -6817,7 +6817,7 @@
         <v>47</v>
       </c>
       <c r="J64" t="n">
-        <v>4.942873477935791</v>
+        <v>3.885893106460571</v>
       </c>
       <c r="K64" t="n">
         <v>66</v>
@@ -6849,10 +6849,10 @@
         <v>39</v>
       </c>
       <c r="T64" t="n">
-        <v>246.5949063301086</v>
+        <v>230.2946786880493</v>
       </c>
       <c r="U64" t="n">
-        <v>251.5390617847443</v>
+        <v>234.1825270652771</v>
       </c>
       <c r="V64" t="inlineStr">
         <is>
@@ -6893,7 +6893,7 @@
         <v>62</v>
       </c>
       <c r="F65" t="n">
-        <v>0.001606225967407227</v>
+        <v>0.001321315765380859</v>
       </c>
       <c r="G65" t="n">
         <v>49</v>
@@ -6905,7 +6905,7 @@
         <v>49</v>
       </c>
       <c r="J65" t="n">
-        <v>5.475486040115356</v>
+        <v>5.583125591278076</v>
       </c>
       <c r="K65" t="n">
         <v>87</v>
@@ -6937,10 +6937,10 @@
         <v>41</v>
       </c>
       <c r="T65" t="n">
-        <v>213.2360548973083</v>
+        <v>199.8180537223816</v>
       </c>
       <c r="U65" t="n">
-        <v>218.7131471633911</v>
+        <v>205.402500629425</v>
       </c>
       <c r="V65" t="inlineStr">
         <is>
@@ -6981,7 +6981,7 @@
         <v>62</v>
       </c>
       <c r="F66" t="n">
-        <v>0.001995563507080078</v>
+        <v>0.001492023468017578</v>
       </c>
       <c r="G66" t="n">
         <v>51</v>
@@ -6993,7 +6993,7 @@
         <v>51</v>
       </c>
       <c r="J66" t="n">
-        <v>3.973000049591064</v>
+        <v>4.190337181091309</v>
       </c>
       <c r="K66" t="n">
         <v>64</v>
@@ -7025,10 +7025,10 @@
         <v>38</v>
       </c>
       <c r="T66" t="n">
-        <v>358.7408716678619</v>
+        <v>354.2173273563385</v>
       </c>
       <c r="U66" t="n">
-        <v>362.7158672809601</v>
+        <v>358.4091565608978</v>
       </c>
       <c r="V66" t="inlineStr">
         <is>
@@ -7069,7 +7069,7 @@
         <v>58</v>
       </c>
       <c r="F67" t="n">
-        <v>0.001418590545654297</v>
+        <v>0.001523494720458984</v>
       </c>
       <c r="G67" t="n">
         <v>49</v>
@@ -7081,7 +7081,7 @@
         <v>49</v>
       </c>
       <c r="J67" t="n">
-        <v>5.562726259231567</v>
+        <v>5.573826313018799</v>
       </c>
       <c r="K67" t="n">
         <v>84</v>
@@ -7113,10 +7113,10 @@
         <v>39</v>
       </c>
       <c r="T67" t="n">
-        <v>247.3467922210693</v>
+        <v>254.5672690868378</v>
       </c>
       <c r="U67" t="n">
-        <v>252.9109370708466</v>
+        <v>260.142618894577</v>
       </c>
       <c r="V67" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         <v>61</v>
       </c>
       <c r="F68" t="n">
-        <v>0.002726078033447266</v>
+        <v>0.001307964324951172</v>
       </c>
       <c r="G68" t="n">
         <v>50</v>
@@ -7169,7 +7169,7 @@
         <v>50</v>
       </c>
       <c r="J68" t="n">
-        <v>6.213391065597534</v>
+        <v>11.62190818786621</v>
       </c>
       <c r="K68" t="n">
         <v>88</v>
@@ -7201,10 +7201,10 @@
         <v>39</v>
       </c>
       <c r="T68" t="n">
-        <v>167.9070084095001</v>
+        <v>180.0540564060211</v>
       </c>
       <c r="U68" t="n">
-        <v>174.1231255531311</v>
+        <v>191.6772725582123</v>
       </c>
       <c r="V68" t="inlineStr">
         <is>
@@ -7245,7 +7245,7 @@
         <v>60</v>
       </c>
       <c r="F69" t="n">
-        <v>0.002372980117797852</v>
+        <v>0.002844095230102539</v>
       </c>
       <c r="G69" t="n">
         <v>44</v>
@@ -7257,7 +7257,7 @@
         <v>44</v>
       </c>
       <c r="J69" t="n">
-        <v>10.88135266304016</v>
+        <v>10.92037606239319</v>
       </c>
       <c r="K69" t="n">
         <v>116</v>
@@ -7289,10 +7289,10 @@
         <v>40</v>
       </c>
       <c r="T69" t="n">
-        <v>228.2792825698853</v>
+        <v>248.622581243515</v>
       </c>
       <c r="U69" t="n">
-        <v>239.1630082130432</v>
+        <v>259.5458014011383</v>
       </c>
       <c r="V69" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
         <v>66</v>
       </c>
       <c r="F70" t="n">
-        <v>0.001785516738891602</v>
+        <v>0.001315116882324219</v>
       </c>
       <c r="G70" t="n">
         <v>50</v>
@@ -7345,7 +7345,7 @@
         <v>50</v>
       </c>
       <c r="J70" t="n">
-        <v>5.670689105987549</v>
+        <v>8.634723663330078</v>
       </c>
       <c r="K70" t="n">
         <v>84</v>
@@ -7377,10 +7377,10 @@
         <v>38</v>
       </c>
       <c r="T70" t="n">
-        <v>373.9893279075623</v>
+        <v>405.5759167671204</v>
       </c>
       <c r="U70" t="n">
-        <v>379.6618025302887</v>
+        <v>414.2119555473328</v>
       </c>
       <c r="V70" t="inlineStr">
         <is>
@@ -7421,7 +7421,7 @@
         <v>66</v>
       </c>
       <c r="F71" t="n">
-        <v>0.002199411392211914</v>
+        <v>0.001315832138061523</v>
       </c>
       <c r="G71" t="n">
         <v>44</v>
@@ -7433,7 +7433,7 @@
         <v>44</v>
       </c>
       <c r="J71" t="n">
-        <v>8.358654022216797</v>
+        <v>9.758319616317749</v>
       </c>
       <c r="K71" t="n">
         <v>132</v>
@@ -7465,10 +7465,10 @@
         <v>37</v>
       </c>
       <c r="T71" t="n">
-        <v>230.1295580863953</v>
+        <v>270.5633101463318</v>
       </c>
       <c r="U71" t="n">
-        <v>238.4904115200043</v>
+        <v>280.3229455947876</v>
       </c>
       <c r="V71" t="inlineStr">
         <is>
@@ -7643,7 +7643,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.624800443649292</v>
+        <v>0.7148253917694092</v>
       </c>
       <c r="M2" t="n">
         <v>500</v>
@@ -7699,7 +7699,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7156004905700684</v>
+        <v>0.7130506038665771</v>
       </c>
       <c r="M3" t="n">
         <v>500</v>
@@ -7755,7 +7755,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6380014419555664</v>
+        <v>0.6269407272338867</v>
       </c>
       <c r="M4" t="n">
         <v>500</v>
@@ -7811,7 +7811,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6063680648803711</v>
+        <v>0.6857600212097168</v>
       </c>
       <c r="M5" t="n">
         <v>500</v>
@@ -7867,7 +7867,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6124095916748047</v>
+        <v>0.6889545917510986</v>
       </c>
       <c r="M6" t="n">
         <v>500</v>
@@ -7923,7 +7923,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6643798351287842</v>
+        <v>0.7694838047027588</v>
       </c>
       <c r="M7" t="n">
         <v>500</v>
@@ -7979,7 +7979,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5690939426422119</v>
+        <v>0.6996982097625732</v>
       </c>
       <c r="M8" t="n">
         <v>500</v>
@@ -8035,7 +8035,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5931298732757568</v>
+        <v>0.6943035125732422</v>
       </c>
       <c r="M9" t="n">
         <v>500</v>
@@ -8091,7 +8091,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6410448551177979</v>
+        <v>0.7941954135894775</v>
       </c>
       <c r="M10" t="n">
         <v>500</v>
@@ -8147,7 +8147,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5688900947570801</v>
+        <v>0.6948974132537842</v>
       </c>
       <c r="M11" t="n">
         <v>500</v>
@@ -8203,7 +8203,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1.209953308105469</v>
+        <v>1.68302845954895</v>
       </c>
       <c r="M12" t="n">
         <v>500</v>
@@ -8259,7 +8259,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>1.324868679046631</v>
+        <v>1.700077772140503</v>
       </c>
       <c r="M13" t="n">
         <v>500</v>
@@ -8315,7 +8315,7 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1.286658763885498</v>
+        <v>1.64783501625061</v>
       </c>
       <c r="M14" t="n">
         <v>500</v>
@@ -8371,7 +8371,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>1.337256908416748</v>
+        <v>1.850628614425659</v>
       </c>
       <c r="M15" t="n">
         <v>500</v>
@@ -8427,7 +8427,7 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>1.41843581199646</v>
+        <v>1.726575374603271</v>
       </c>
       <c r="M16" t="n">
         <v>500</v>
@@ -8483,7 +8483,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>1.210504293441772</v>
+        <v>1.499370813369751</v>
       </c>
       <c r="M17" t="n">
         <v>500</v>
@@ -8539,7 +8539,7 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>1.407422780990601</v>
+        <v>1.85375452041626</v>
       </c>
       <c r="M18" t="n">
         <v>500</v>
@@ -8595,7 +8595,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>1.268229246139526</v>
+        <v>1.614604949951172</v>
       </c>
       <c r="M19" t="n">
         <v>500</v>
@@ -8651,7 +8651,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>1.291438102722168</v>
+        <v>1.630741834640503</v>
       </c>
       <c r="M20" t="n">
         <v>500</v>
@@ -8707,7 +8707,7 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>1.265780925750732</v>
+        <v>1.623961448669434</v>
       </c>
       <c r="M21" t="n">
         <v>500</v>
@@ -8763,7 +8763,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1.659703016281128</v>
+        <v>2.192342281341553</v>
       </c>
       <c r="M22" t="n">
         <v>500</v>
@@ -8819,7 +8819,7 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>1.783647060394287</v>
+        <v>2.517016887664795</v>
       </c>
       <c r="M23" t="n">
         <v>500</v>
@@ -8875,7 +8875,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>1.891098022460938</v>
+        <v>2.445166349411011</v>
       </c>
       <c r="M24" t="n">
         <v>500</v>
@@ -8931,7 +8931,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>1.691244602203369</v>
+        <v>2.265771865844727</v>
       </c>
       <c r="M25" t="n">
         <v>500</v>
@@ -8987,7 +8987,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>1.777453184127808</v>
+        <v>2.335699319839478</v>
       </c>
       <c r="M26" t="n">
         <v>500</v>
@@ -9043,7 +9043,7 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>1.772819995880127</v>
+        <v>2.376081705093384</v>
       </c>
       <c r="M27" t="n">
         <v>500</v>
@@ -9099,7 +9099,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>1.916248798370361</v>
+        <v>2.512481689453125</v>
       </c>
       <c r="M28" t="n">
         <v>500</v>
@@ -9155,7 +9155,7 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>1.743336200714111</v>
+        <v>2.144961833953857</v>
       </c>
       <c r="M29" t="n">
         <v>500</v>
@@ -9211,7 +9211,7 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>1.784942626953125</v>
+        <v>2.324721097946167</v>
       </c>
       <c r="M30" t="n">
         <v>500</v>
@@ -9267,7 +9267,7 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>1.887743234634399</v>
+        <v>2.33649468421936</v>
       </c>
       <c r="M31" t="n">
         <v>500</v>
@@ -9323,7 +9323,7 @@
         <v>9</v>
       </c>
       <c r="L32" t="n">
-        <v>26.69189119338989</v>
+        <v>39.22724962234497</v>
       </c>
       <c r="M32" t="n">
         <v>1130</v>
@@ -9379,7 +9379,7 @@
         <v>9</v>
       </c>
       <c r="L33" t="n">
-        <v>19.51586365699768</v>
+        <v>29.58467650413513</v>
       </c>
       <c r="M33" t="n">
         <v>842</v>
@@ -9435,7 +9435,7 @@
         <v>10</v>
       </c>
       <c r="L34" t="n">
-        <v>16.07514715194702</v>
+        <v>24.61968851089478</v>
       </c>
       <c r="M34" t="n">
         <v>699</v>
@@ -9491,7 +9491,7 @@
         <v>9</v>
       </c>
       <c r="L35" t="n">
-        <v>13.54414629936218</v>
+        <v>19.97590231895447</v>
       </c>
       <c r="M35" t="n">
         <v>600</v>
@@ -9547,7 +9547,7 @@
         <v>9</v>
       </c>
       <c r="L36" t="n">
-        <v>21.19950008392334</v>
+        <v>30.57473802566528</v>
       </c>
       <c r="M36" t="n">
         <v>904</v>
@@ -9603,7 +9603,7 @@
         <v>9</v>
       </c>
       <c r="L37" t="n">
-        <v>23.70487785339355</v>
+        <v>35.10482335090637</v>
       </c>
       <c r="M37" t="n">
         <v>981</v>
@@ -9659,7 +9659,7 @@
         <v>9</v>
       </c>
       <c r="L38" t="n">
-        <v>21.38955283164978</v>
+        <v>31.64168238639832</v>
       </c>
       <c r="M38" t="n">
         <v>963</v>
@@ -9715,7 +9715,7 @@
         <v>9</v>
       </c>
       <c r="L39" t="n">
-        <v>17.1313488483429</v>
+        <v>25.88877987861633</v>
       </c>
       <c r="M39" t="n">
         <v>757</v>
@@ -9771,7 +9771,7 @@
         <v>9</v>
       </c>
       <c r="L40" t="n">
-        <v>28.320481300354</v>
+        <v>43.41889977455139</v>
       </c>
       <c r="M40" t="n">
         <v>1147</v>
@@ -9827,7 +9827,7 @@
         <v>9</v>
       </c>
       <c r="L41" t="n">
-        <v>25.28454303741455</v>
+        <v>32.1569197177887</v>
       </c>
       <c r="M41" t="n">
         <v>1182</v>
@@ -9883,7 +9883,7 @@
         <v>20</v>
       </c>
       <c r="L42" t="n">
-        <v>55.13903141021729</v>
+        <v>56.31191802024841</v>
       </c>
       <c r="M42" t="n">
         <v>913</v>
@@ -9939,7 +9939,7 @@
         <v>20</v>
       </c>
       <c r="L43" t="n">
-        <v>60.85281467437744</v>
+        <v>61.94121789932251</v>
       </c>
       <c r="M43" t="n">
         <v>775</v>
@@ -9995,7 +9995,7 @@
         <v>20</v>
       </c>
       <c r="L44" t="n">
-        <v>39.44452929496765</v>
+        <v>40.77013659477234</v>
       </c>
       <c r="M44" t="n">
         <v>573</v>
@@ -10051,7 +10051,7 @@
         <v>19</v>
       </c>
       <c r="L45" t="n">
-        <v>70.94095158576965</v>
+        <v>72.76348805427551</v>
       </c>
       <c r="M45" t="n">
         <v>1010</v>
@@ -10107,7 +10107,7 @@
         <v>20</v>
       </c>
       <c r="L46" t="n">
-        <v>63.33185529708862</v>
+        <v>48.28197240829468</v>
       </c>
       <c r="M46" t="n">
         <v>681</v>
@@ -10163,7 +10163,7 @@
         <v>20</v>
       </c>
       <c r="L47" t="n">
-        <v>72.22267270088196</v>
+        <v>66.96747064590454</v>
       </c>
       <c r="M47" t="n">
         <v>925</v>
@@ -10219,7 +10219,7 @@
         <v>19</v>
       </c>
       <c r="L48" t="n">
-        <v>91.30044651031494</v>
+        <v>76.89169049263</v>
       </c>
       <c r="M48" t="n">
         <v>1075</v>
@@ -10275,7 +10275,7 @@
         <v>20</v>
       </c>
       <c r="L49" t="n">
-        <v>78.05465722084045</v>
+        <v>78.91547346115112</v>
       </c>
       <c r="M49" t="n">
         <v>929</v>
@@ -10331,7 +10331,7 @@
         <v>19</v>
       </c>
       <c r="L50" t="n">
-        <v>73.07584238052368</v>
+        <v>84.49457049369812</v>
       </c>
       <c r="M50" t="n">
         <v>884</v>
@@ -10387,7 +10387,7 @@
         <v>21</v>
       </c>
       <c r="L51" t="n">
-        <v>45.08503603935242</v>
+        <v>54.05926036834717</v>
       </c>
       <c r="M51" t="n">
         <v>532</v>
@@ -10443,7 +10443,7 @@
         <v>34</v>
       </c>
       <c r="L52" t="n">
-        <v>148.7658965587616</v>
+        <v>181.0873084068298</v>
       </c>
       <c r="M52" t="n">
         <v>961</v>
@@ -10499,7 +10499,7 @@
         <v>36</v>
       </c>
       <c r="L53" t="n">
-        <v>100.6322181224823</v>
+        <v>111.8289468288422</v>
       </c>
       <c r="M53" t="n">
         <v>549</v>
@@ -10555,7 +10555,7 @@
         <v>32</v>
       </c>
       <c r="L54" t="n">
-        <v>226.8178315162659</v>
+        <v>201.4471638202667</v>
       </c>
       <c r="M54" t="n">
         <v>1125</v>
@@ -10611,7 +10611,7 @@
         <v>35</v>
       </c>
       <c r="L55" t="n">
-        <v>134.5764470100403</v>
+        <v>145.4961667060852</v>
       </c>
       <c r="M55" t="n">
         <v>775</v>
@@ -10667,7 +10667,7 @@
         <v>33</v>
       </c>
       <c r="L56" t="n">
-        <v>119.2966840267181</v>
+        <v>189.0848925113678</v>
       </c>
       <c r="M56" t="n">
         <v>988</v>
@@ -10723,7 +10723,7 @@
         <v>38</v>
       </c>
       <c r="L57" t="n">
-        <v>72.36353182792664</v>
+        <v>99.97208905220032</v>
       </c>
       <c r="M57" t="n">
         <v>593</v>
@@ -10779,7 +10779,7 @@
         <v>38</v>
       </c>
       <c r="L58" t="n">
-        <v>73.40750288963318</v>
+        <v>88.6357409954071</v>
       </c>
       <c r="M58" t="n">
         <v>510</v>
@@ -10835,7 +10835,7 @@
         <v>33</v>
       </c>
       <c r="L59" t="n">
-        <v>180.5149443149567</v>
+        <v>217.1243646144867</v>
       </c>
       <c r="M59" t="n">
         <v>1124</v>
@@ -10891,7 +10891,7 @@
         <v>33</v>
       </c>
       <c r="L60" t="n">
-        <v>270.9640567302704</v>
+        <v>346.1360051631927</v>
       </c>
       <c r="M60" t="n">
         <v>1543</v>
@@ -10947,7 +10947,7 @@
         <v>34</v>
       </c>
       <c r="L61" t="n">
-        <v>200.8792588710785</v>
+        <v>493.0264613628387</v>
       </c>
       <c r="M61" t="n">
         <v>1427</v>
@@ -11003,14 +11003,14 @@
         <v>39</v>
       </c>
       <c r="L62" t="n">
-        <v>342.6690044403076</v>
+        <v>600.4185683727264</v>
       </c>
       <c r="M62" t="n">
-        <v>1608</v>
+        <v>1298</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>no_imp_lim</t>
+          <t>t_lim</t>
         </is>
       </c>
       <c r="O62" t="b">
@@ -11059,7 +11059,7 @@
         <v>39</v>
       </c>
       <c r="L63" t="n">
-        <v>270.610095500946</v>
+        <v>243.6602087020874</v>
       </c>
       <c r="M63" t="n">
         <v>1350</v>
@@ -11115,7 +11115,7 @@
         <v>39</v>
       </c>
       <c r="L64" t="n">
-        <v>246.5949063301086</v>
+        <v>230.2946786880493</v>
       </c>
       <c r="M64" t="n">
         <v>1265</v>
@@ -11171,7 +11171,7 @@
         <v>41</v>
       </c>
       <c r="L65" t="n">
-        <v>213.2360548973083</v>
+        <v>199.8180537223816</v>
       </c>
       <c r="M65" t="n">
         <v>1027</v>
@@ -11227,7 +11227,7 @@
         <v>38</v>
       </c>
       <c r="L66" t="n">
-        <v>358.7408716678619</v>
+        <v>354.2173273563385</v>
       </c>
       <c r="M66" t="n">
         <v>2000</v>
@@ -11283,7 +11283,7 @@
         <v>39</v>
       </c>
       <c r="L67" t="n">
-        <v>247.3467922210693</v>
+        <v>254.5672690868378</v>
       </c>
       <c r="M67" t="n">
         <v>1231</v>
@@ -11339,7 +11339,7 @@
         <v>39</v>
       </c>
       <c r="L68" t="n">
-        <v>167.9070084095001</v>
+        <v>180.0540564060211</v>
       </c>
       <c r="M68" t="n">
         <v>925</v>
@@ -11395,7 +11395,7 @@
         <v>40</v>
       </c>
       <c r="L69" t="n">
-        <v>228.2792825698853</v>
+        <v>248.622581243515</v>
       </c>
       <c r="M69" t="n">
         <v>1202</v>
@@ -11451,7 +11451,7 @@
         <v>38</v>
       </c>
       <c r="L70" t="n">
-        <v>373.9893279075623</v>
+        <v>405.5759167671204</v>
       </c>
       <c r="M70" t="n">
         <v>2000</v>
@@ -11507,7 +11507,7 @@
         <v>37</v>
       </c>
       <c r="L71" t="n">
-        <v>230.1295580863953</v>
+        <v>270.5633101463318</v>
       </c>
       <c r="M71" t="n">
         <v>1351</v>
@@ -11708,7 +11708,7 @@
         <v>10</v>
       </c>
       <c r="I2" t="n">
-        <v>0.623</v>
+        <v>0.674</v>
       </c>
       <c r="J2" t="n">
         <v>31.6</v>
@@ -11733,10 +11733,10 @@
         <v>10</v>
       </c>
       <c r="P2" t="n">
-        <v>3.855</v>
+        <v>4.407</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.232</v>
+        <v>3.733</v>
       </c>
       <c r="R2" t="n">
         <v>561.6</v>
@@ -11793,7 +11793,7 @@
         <v>16</v>
       </c>
       <c r="I3" t="n">
-        <v>1.493</v>
+        <v>1.567</v>
       </c>
       <c r="J3" t="n">
         <v>51.6</v>
@@ -11818,10 +11818,10 @@
         <v>16</v>
       </c>
       <c r="P3" t="n">
-        <v>8.199999999999999</v>
+        <v>9.446</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.706</v>
+        <v>7.879</v>
       </c>
       <c r="R3" t="n">
         <v>641.7</v>
@@ -11878,7 +11878,7 @@
         <v>45</v>
       </c>
       <c r="I4" t="n">
-        <v>7.782</v>
+        <v>6.705</v>
       </c>
       <c r="J4" t="n">
         <v>84.5</v>
@@ -11903,10 +11903,10 @@
         <v>38</v>
       </c>
       <c r="P4" t="n">
-        <v>316.599</v>
+        <v>270.633</v>
       </c>
       <c r="Q4" t="n">
-        <v>308.815</v>
+        <v>263.926</v>
       </c>
       <c r="R4" t="n">
         <v>1311.9</v>
@@ -11951,7 +11951,7 @@
         <v>73</v>
       </c>
       <c r="E5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F5" t="n">
         <v>64.09999999999999</v>
@@ -11963,7 +11963,7 @@
         <v>59</v>
       </c>
       <c r="I5" t="n">
-        <v>13.52</v>
+        <v>8.266</v>
       </c>
       <c r="J5" t="n">
         <v>96.8</v>
@@ -11979,22 +11979,22 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="N5" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="O5" t="n">
         <v>48</v>
       </c>
       <c r="P5" t="n">
-        <v>470.772</v>
+        <v>426.197</v>
       </c>
       <c r="Q5" t="n">
-        <v>457.249</v>
+        <v>417.929</v>
       </c>
       <c r="R5" t="n">
-        <v>1216.2</v>
+        <v>1321.1</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -12003,12 +12003,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>-35.10%</t>
+          <t>-35.23%</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>-19.51%</t>
+          <t>-19.66%</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -12017,7 +12017,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
     </row>
   </sheetData>
@@ -12043,7 +12043,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
@@ -12213,7 +12213,7 @@
         <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0003662109375</v>
+        <v>0.0003073215484619141</v>
       </c>
       <c r="G2" t="n">
         <v>11</v>
@@ -12225,7 +12225,7 @@
         <v>11</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7858119010925293</v>
+        <v>0.848130464553833</v>
       </c>
       <c r="K2" t="n">
         <v>42</v>
@@ -12257,10 +12257,10 @@
         <v>10</v>
       </c>
       <c r="T2" t="n">
-        <v>2.564436674118042</v>
+        <v>2.652289390563965</v>
       </c>
       <c r="U2" t="n">
-        <v>3.350614786148071</v>
+        <v>3.50072717666626</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -12303,7 +12303,7 @@
         <v>13</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0002434253692626953</v>
+        <v>0.0002589225769042969</v>
       </c>
       <c r="G3" t="n">
         <v>11</v>
@@ -12315,7 +12315,7 @@
         <v>11</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5666849613189697</v>
+        <v>0.5901727676391602</v>
       </c>
       <c r="K3" t="n">
         <v>31</v>
@@ -12347,10 +12347,10 @@
         <v>10</v>
       </c>
       <c r="T3" t="n">
-        <v>2.71745777130127</v>
+        <v>3.514975547790527</v>
       </c>
       <c r="U3" t="n">
-        <v>3.284386157989502</v>
+        <v>4.105407238006592</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
@@ -12393,7 +12393,7 @@
         <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0002527236938476562</v>
+        <v>0.0004041194915771484</v>
       </c>
       <c r="G4" t="n">
         <v>11</v>
@@ -12405,7 +12405,7 @@
         <v>11</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5131340026855469</v>
+        <v>0.6771183013916016</v>
       </c>
       <c r="K4" t="n">
         <v>27</v>
@@ -12437,10 +12437,10 @@
         <v>10</v>
       </c>
       <c r="T4" t="n">
-        <v>8.255967140197754</v>
+        <v>4.19107723236084</v>
       </c>
       <c r="U4" t="n">
-        <v>8.769353866577148</v>
+        <v>4.868599653244019</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -12483,7 +12483,7 @@
         <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0002484321594238281</v>
+        <v>0.0002512931823730469</v>
       </c>
       <c r="G5" t="n">
         <v>10</v>
@@ -12495,7 +12495,7 @@
         <v>10</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6598305702209473</v>
+        <v>0.7043805122375488</v>
       </c>
       <c r="K5" t="n">
         <v>34</v>
@@ -12527,10 +12527,10 @@
         <v>10</v>
       </c>
       <c r="T5" t="n">
-        <v>2.769766569137573</v>
+        <v>3.228170871734619</v>
       </c>
       <c r="U5" t="n">
-        <v>3.429845571517944</v>
+        <v>3.932802677154541</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -12573,7 +12573,7 @@
         <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0003232955932617188</v>
+        <v>0.0005104541778564453</v>
       </c>
       <c r="G6" t="n">
         <v>11</v>
@@ -12585,7 +12585,7 @@
         <v>11</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4509818553924561</v>
+        <v>0.6542770862579346</v>
       </c>
       <c r="K6" t="n">
         <v>25</v>
@@ -12617,10 +12617,10 @@
         <v>10</v>
       </c>
       <c r="T6" t="n">
-        <v>3.657449245452881</v>
+        <v>3.953996658325195</v>
       </c>
       <c r="U6" t="n">
-        <v>4.108754396438599</v>
+        <v>4.608784198760986</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -12663,7 +12663,7 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>0.000339508056640625</v>
+        <v>0.0002455711364746094</v>
       </c>
       <c r="G7" t="n">
         <v>10</v>
@@ -12675,7 +12675,7 @@
         <v>10</v>
       </c>
       <c r="J7" t="n">
-        <v>0.8482382297515869</v>
+        <v>0.8763797283172607</v>
       </c>
       <c r="K7" t="n">
         <v>39</v>
@@ -12707,10 +12707,10 @@
         <v>10</v>
       </c>
       <c r="T7" t="n">
-        <v>2.199610233306885</v>
+        <v>8.113522291183472</v>
       </c>
       <c r="U7" t="n">
-        <v>3.048187971115112</v>
+        <v>8.990147590637207</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -12753,7 +12753,7 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0002558231353759766</v>
+        <v>0.0002677440643310547</v>
       </c>
       <c r="G8" t="n">
         <v>10</v>
@@ -12765,7 +12765,7 @@
         <v>10</v>
       </c>
       <c r="J8" t="n">
-        <v>0.545180082321167</v>
+        <v>0.5748467445373535</v>
       </c>
       <c r="K8" t="n">
         <v>28</v>
@@ -12797,10 +12797,10 @@
         <v>10</v>
       </c>
       <c r="T8" t="n">
-        <v>2.359295606613159</v>
+        <v>2.572837829589844</v>
       </c>
       <c r="U8" t="n">
-        <v>2.904731512069702</v>
+        <v>3.147952318191528</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
@@ -12843,7 +12843,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0002527236938476562</v>
+        <v>0.0002961158752441406</v>
       </c>
       <c r="G9" t="n">
         <v>10</v>
@@ -12855,7 +12855,7 @@
         <v>10</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7983150482177734</v>
+        <v>0.7032701969146729</v>
       </c>
       <c r="K9" t="n">
         <v>34</v>
@@ -12887,10 +12887,10 @@
         <v>10</v>
       </c>
       <c r="T9" t="n">
-        <v>3.043267726898193</v>
+        <v>4.035722970962524</v>
       </c>
       <c r="U9" t="n">
-        <v>3.841835498809814</v>
+        <v>4.739289283752441</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
@@ -12933,7 +12933,7 @@
         <v>13</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0002498626708984375</v>
+        <v>0.0002620220184326172</v>
       </c>
       <c r="G10" t="n">
         <v>11</v>
@@ -12945,7 +12945,7 @@
         <v>11</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4992704391479492</v>
+        <v>0.5344784259796143</v>
       </c>
       <c r="K10" t="n">
         <v>27</v>
@@ -12977,10 +12977,10 @@
         <v>10</v>
       </c>
       <c r="T10" t="n">
-        <v>2.620037317276001</v>
+        <v>2.831363439559937</v>
       </c>
       <c r="U10" t="n">
-        <v>3.119557619094849</v>
+        <v>3.366103887557983</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -13023,7 +13023,7 @@
         <v>13</v>
       </c>
       <c r="F11" t="n">
-        <v>0.000293731689453125</v>
+        <v>0.0002570152282714844</v>
       </c>
       <c r="G11" t="n">
         <v>11</v>
@@ -13035,7 +13035,7 @@
         <v>11</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5595407485961914</v>
+        <v>0.572451114654541</v>
       </c>
       <c r="K11" t="n">
         <v>29</v>
@@ -13067,10 +13067,10 @@
         <v>10</v>
       </c>
       <c r="T11" t="n">
-        <v>2.135944366455078</v>
+        <v>2.233396768569946</v>
       </c>
       <c r="U11" t="n">
-        <v>2.695778846740723</v>
+        <v>2.806104898452759</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
@@ -13113,7 +13113,7 @@
         <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0004088878631591797</v>
+        <v>0.0004084110260009766</v>
       </c>
       <c r="G12" t="n">
         <v>20</v>
@@ -13125,7 +13125,7 @@
         <v>20</v>
       </c>
       <c r="J12" t="n">
-        <v>1.223306179046631</v>
+        <v>1.304376602172852</v>
       </c>
       <c r="K12" t="n">
         <v>45</v>
@@ -13157,10 +13157,10 @@
         <v>18</v>
       </c>
       <c r="T12" t="n">
-        <v>7.197542905807495</v>
+        <v>8.463103532791138</v>
       </c>
       <c r="U12" t="n">
-        <v>8.421257972717285</v>
+        <v>9.76788854598999</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -13203,7 +13203,7 @@
         <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0004932880401611328</v>
+        <v>0.0003845691680908203</v>
       </c>
       <c r="G13" t="n">
         <v>19</v>
@@ -13215,7 +13215,7 @@
         <v>19</v>
       </c>
       <c r="J13" t="n">
-        <v>1.009407758712769</v>
+        <v>1.038631677627563</v>
       </c>
       <c r="K13" t="n">
         <v>37</v>
@@ -13247,10 +13247,10 @@
         <v>18</v>
       </c>
       <c r="T13" t="n">
-        <v>4.722747564315796</v>
+        <v>5.842691659927368</v>
       </c>
       <c r="U13" t="n">
-        <v>5.732648611068726</v>
+        <v>6.881707906723022</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         <v>26</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0004093647003173828</v>
+        <v>0.00040435791015625</v>
       </c>
       <c r="G14" t="n">
         <v>19</v>
@@ -13305,7 +13305,7 @@
         <v>19</v>
       </c>
       <c r="J14" t="n">
-        <v>1.134420394897461</v>
+        <v>1.240294694900513</v>
       </c>
       <c r="K14" t="n">
         <v>43</v>
@@ -13337,10 +13337,10 @@
         <v>16</v>
       </c>
       <c r="T14" t="n">
-        <v>7.404346704483032</v>
+        <v>8.529135704040527</v>
       </c>
       <c r="U14" t="n">
-        <v>8.539176464080811</v>
+        <v>9.769834756851196</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
@@ -13383,7 +13383,7 @@
         <v>26</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0004322528839111328</v>
+        <v>0.0003993511199951172</v>
       </c>
       <c r="G15" t="n">
         <v>16</v>
@@ -13395,7 +13395,7 @@
         <v>16</v>
       </c>
       <c r="J15" t="n">
-        <v>2.239801168441772</v>
+        <v>2.354054689407349</v>
       </c>
       <c r="K15" t="n">
         <v>77</v>
@@ -13427,10 +13427,10 @@
         <v>16</v>
       </c>
       <c r="T15" t="n">
-        <v>4.710891485214233</v>
+        <v>5.819690942764282</v>
       </c>
       <c r="U15" t="n">
-        <v>6.951124906539917</v>
+        <v>8.174144983291626</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
@@ -13473,7 +13473,7 @@
         <v>25</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0003895759582519531</v>
+        <v>0.0003917217254638672</v>
       </c>
       <c r="G16" t="n">
         <v>18</v>
@@ -13485,7 +13485,7 @@
         <v>18</v>
       </c>
       <c r="J16" t="n">
-        <v>1.424978971481323</v>
+        <v>1.511151075363159</v>
       </c>
       <c r="K16" t="n">
         <v>49</v>
@@ -13517,10 +13517,10 @@
         <v>17</v>
       </c>
       <c r="T16" t="n">
-        <v>11.27451801300049</v>
+        <v>12.38631439208984</v>
       </c>
       <c r="U16" t="n">
-        <v>12.69988656044006</v>
+        <v>13.89785718917847</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
@@ -13563,7 +13563,7 @@
         <v>25</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0003819465637207031</v>
+        <v>0.0003917217254638672</v>
       </c>
       <c r="G17" t="n">
         <v>18</v>
@@ -13575,7 +13575,7 @@
         <v>18</v>
       </c>
       <c r="J17" t="n">
-        <v>1.304403305053711</v>
+        <v>1.448296070098877</v>
       </c>
       <c r="K17" t="n">
         <v>42</v>
@@ -13607,10 +13607,10 @@
         <v>18</v>
       </c>
       <c r="T17" t="n">
-        <v>6.062460660934448</v>
+        <v>7.169698715209961</v>
       </c>
       <c r="U17" t="n">
-        <v>7.36724591255188</v>
+        <v>8.618386507034302</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
@@ -13653,7 +13653,7 @@
         <v>27</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0003554821014404297</v>
+        <v>0.0003566741943359375</v>
       </c>
       <c r="G18" t="n">
         <v>18</v>
@@ -13665,7 +13665,7 @@
         <v>18</v>
       </c>
       <c r="J18" t="n">
-        <v>2.13327431678772</v>
+        <v>2.214152336120605</v>
       </c>
       <c r="K18" t="n">
         <v>67</v>
@@ -13697,10 +13697,10 @@
         <v>17</v>
       </c>
       <c r="T18" t="n">
-        <v>5.887769937515259</v>
+        <v>7.005539655685425</v>
       </c>
       <c r="U18" t="n">
-        <v>8.021399736404419</v>
+        <v>9.220048666000366</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
         <v>25</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0004742145538330078</v>
+        <v>0.00035858154296875</v>
       </c>
       <c r="G19" t="n">
         <v>19</v>
@@ -13755,7 +13755,7 @@
         <v>19</v>
       </c>
       <c r="J19" t="n">
-        <v>2.133487462997437</v>
+        <v>2.163874387741089</v>
       </c>
       <c r="K19" t="n">
         <v>70</v>
@@ -13787,10 +13787,10 @@
         <v>18</v>
       </c>
       <c r="T19" t="n">
-        <v>6.479783535003662</v>
+        <v>7.740480661392212</v>
       </c>
       <c r="U19" t="n">
-        <v>8.613745212554932</v>
+        <v>9.90471363067627</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -13833,7 +13833,7 @@
         <v>25</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0003664493560791016</v>
+        <v>0.0006325244903564453</v>
       </c>
       <c r="G20" t="n">
         <v>21</v>
@@ -13845,7 +13845,7 @@
         <v>21</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5657036304473877</v>
+        <v>0.5898687839508057</v>
       </c>
       <c r="K20" t="n">
         <v>24</v>
@@ -13877,10 +13877,10 @@
         <v>17</v>
       </c>
       <c r="T20" t="n">
-        <v>9.089521169662476</v>
+        <v>10.49940276145935</v>
       </c>
       <c r="U20" t="n">
-        <v>9.655591249465942</v>
+        <v>11.08990406990051</v>
       </c>
       <c r="V20" t="inlineStr">
         <is>
@@ -13923,7 +13923,7 @@
         <v>24</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0003287792205810547</v>
+        <v>0.0003299713134765625</v>
       </c>
       <c r="G21" t="n">
         <v>18</v>
@@ -13935,7 +13935,7 @@
         <v>18</v>
       </c>
       <c r="J21" t="n">
-        <v>1.765857696533203</v>
+        <v>1.806029796600342</v>
       </c>
       <c r="K21" t="n">
         <v>62</v>
@@ -13967,10 +13967,10 @@
         <v>18</v>
       </c>
       <c r="T21" t="n">
-        <v>4.228868246078491</v>
+        <v>5.332628011703491</v>
       </c>
       <c r="U21" t="n">
-        <v>5.995054721832275</v>
+        <v>7.13898777961731</v>
       </c>
       <c r="V21" t="inlineStr">
         <is>
@@ -14013,7 +14013,7 @@
         <v>59</v>
       </c>
       <c r="F22" t="n">
-        <v>0.001266717910766602</v>
+        <v>0.001304864883422852</v>
       </c>
       <c r="G22" t="n">
         <v>52</v>
@@ -14025,7 +14025,7 @@
         <v>52</v>
       </c>
       <c r="J22" t="n">
-        <v>2.893081188201904</v>
+        <v>3.046880006790161</v>
       </c>
       <c r="K22" t="n">
         <v>53</v>
@@ -14057,10 +14057,10 @@
         <v>41</v>
       </c>
       <c r="T22" t="n">
-        <v>488.5111601352692</v>
+        <v>337.8674705028534</v>
       </c>
       <c r="U22" t="n">
-        <v>491.4055080413818</v>
+        <v>340.915655374527</v>
       </c>
       <c r="V22" t="inlineStr">
         <is>
@@ -14103,7 +14103,7 @@
         <v>65</v>
       </c>
       <c r="F23" t="n">
-        <v>0.003899335861206055</v>
+        <v>0.001749992370605469</v>
       </c>
       <c r="G23" t="n">
         <v>46</v>
@@ -14115,7 +14115,7 @@
         <v>46</v>
       </c>
       <c r="J23" t="n">
-        <v>8.768959522247314</v>
+        <v>13.40820956230164</v>
       </c>
       <c r="K23" t="n">
         <v>113</v>
@@ -14147,10 +14147,10 @@
         <v>46</v>
       </c>
       <c r="T23" t="n">
-        <v>134.8803567886353</v>
+        <v>106.4561235904694</v>
       </c>
       <c r="U23" t="n">
-        <v>143.6532156467438</v>
+        <v>119.8660831451416</v>
       </c>
       <c r="V23" t="inlineStr">
         <is>
@@ -14193,7 +14193,7 @@
         <v>65</v>
       </c>
       <c r="F24" t="n">
-        <v>0.001549720764160156</v>
+        <v>0.001624822616577148</v>
       </c>
       <c r="G24" t="n">
         <v>46</v>
@@ -14205,7 +14205,7 @@
         <v>46</v>
       </c>
       <c r="J24" t="n">
-        <v>6.321918725967407</v>
+        <v>6.909044742584229</v>
       </c>
       <c r="K24" t="n">
         <v>77</v>
@@ -14237,10 +14237,10 @@
         <v>39</v>
       </c>
       <c r="T24" t="n">
-        <v>393.8975789546967</v>
+        <v>361.5050694942474</v>
       </c>
       <c r="U24" t="n">
-        <v>400.2210474014282</v>
+        <v>368.4157390594482</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -14283,7 +14283,7 @@
         <v>62</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0015411376953125</v>
+        <v>0.001250267028808594</v>
       </c>
       <c r="G25" t="n">
         <v>46</v>
@@ -14295,7 +14295,7 @@
         <v>46</v>
       </c>
       <c r="J25" t="n">
-        <v>15.53117680549622</v>
+        <v>4.916542768478394</v>
       </c>
       <c r="K25" t="n">
         <v>81</v>
@@ -14327,10 +14327,10 @@
         <v>39</v>
       </c>
       <c r="T25" t="n">
-        <v>174.9462289810181</v>
+        <v>168.392587184906</v>
       </c>
       <c r="U25" t="n">
-        <v>190.4789469242096</v>
+        <v>173.3103802204132</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
@@ -14373,7 +14373,7 @@
         <v>64</v>
       </c>
       <c r="F26" t="n">
-        <v>0.001525402069091797</v>
+        <v>0.001287937164306641</v>
       </c>
       <c r="G26" t="n">
         <v>51</v>
@@ -14385,7 +14385,7 @@
         <v>51</v>
       </c>
       <c r="J26" t="n">
-        <v>3.450268507003784</v>
+        <v>3.01085638999939</v>
       </c>
       <c r="K26" t="n">
         <v>53</v>
@@ -14417,10 +14417,10 @@
         <v>41</v>
       </c>
       <c r="T26" t="n">
-        <v>273.1687104701996</v>
+        <v>246.4103243350983</v>
       </c>
       <c r="U26" t="n">
-        <v>276.6205043792725</v>
+        <v>249.422468662262</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
@@ -14463,7 +14463,7 @@
         <v>58</v>
       </c>
       <c r="F27" t="n">
-        <v>0.001463174819946289</v>
+        <v>0.001398086547851562</v>
       </c>
       <c r="G27" t="n">
         <v>46</v>
@@ -14475,7 +14475,7 @@
         <v>46</v>
       </c>
       <c r="J27" t="n">
-        <v>8.555516958236694</v>
+        <v>11.75625538825989</v>
       </c>
       <c r="K27" t="n">
         <v>117</v>
@@ -14507,10 +14507,10 @@
         <v>39</v>
       </c>
       <c r="T27" t="n">
-        <v>321.7855217456818</v>
+        <v>290.6666617393494</v>
       </c>
       <c r="U27" t="n">
-        <v>330.3425018787384</v>
+        <v>302.4243152141571</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
@@ -14553,7 +14553,7 @@
         <v>60</v>
       </c>
       <c r="F28" t="n">
-        <v>0.001400232315063477</v>
+        <v>0.001306295394897461</v>
       </c>
       <c r="G28" t="n">
         <v>45</v>
@@ -14565,7 +14565,7 @@
         <v>45</v>
       </c>
       <c r="J28" t="n">
-        <v>18.69664239883423</v>
+        <v>11.04488229751587</v>
       </c>
       <c r="K28" t="n">
         <v>146</v>
@@ -14597,10 +14597,10 @@
         <v>43</v>
       </c>
       <c r="T28" t="n">
-        <v>102.5393631458282</v>
+        <v>98.49638175964355</v>
       </c>
       <c r="U28" t="n">
-        <v>121.2374057769775</v>
+        <v>109.5425703525543</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
@@ -14643,7 +14643,7 @@
         <v>61</v>
       </c>
       <c r="F29" t="n">
-        <v>0.001384735107421875</v>
+        <v>0.001969575881958008</v>
       </c>
       <c r="G29" t="n">
         <v>52</v>
@@ -14655,7 +14655,7 @@
         <v>52</v>
       </c>
       <c r="J29" t="n">
-        <v>4.433563709259033</v>
+        <v>4.291795969009399</v>
       </c>
       <c r="K29" t="n">
         <v>66</v>
@@ -14687,10 +14687,10 @@
         <v>41</v>
       </c>
       <c r="T29" t="n">
-        <v>375.0543942451477</v>
+        <v>341.0409514904022</v>
       </c>
       <c r="U29" t="n">
-        <v>379.4893426895142</v>
+        <v>345.3347170352936</v>
       </c>
       <c r="V29" t="inlineStr">
         <is>
@@ -14733,7 +14733,7 @@
         <v>65</v>
       </c>
       <c r="F30" t="n">
-        <v>0.001385688781738281</v>
+        <v>0.003026723861694336</v>
       </c>
       <c r="G30" t="n">
         <v>50</v>
@@ -14745,7 +14745,7 @@
         <v>50</v>
       </c>
       <c r="J30" t="n">
-        <v>5.224385738372803</v>
+        <v>4.691082000732422</v>
       </c>
       <c r="K30" t="n">
         <v>73</v>
@@ -14777,10 +14777,10 @@
         <v>38</v>
       </c>
       <c r="T30" t="n">
-        <v>515.514933347702</v>
+        <v>418.7113404273987</v>
       </c>
       <c r="U30" t="n">
-        <v>520.7407047748566</v>
+        <v>423.4054491519928</v>
       </c>
       <c r="V30" t="inlineStr">
         <is>
@@ -14823,7 +14823,7 @@
         <v>66</v>
       </c>
       <c r="F31" t="n">
-        <v>0.001429557800292969</v>
+        <v>0.001607179641723633</v>
       </c>
       <c r="G31" t="n">
         <v>50</v>
@@ -14835,7 +14835,7 @@
         <v>50</v>
       </c>
       <c r="J31" t="n">
-        <v>3.946110725402832</v>
+        <v>3.978266477584839</v>
       </c>
       <c r="K31" t="n">
         <v>66</v>
@@ -14867,10 +14867,10 @@
         <v>40</v>
       </c>
       <c r="T31" t="n">
-        <v>307.8504438400269</v>
+        <v>269.7169692516327</v>
       </c>
       <c r="U31" t="n">
-        <v>311.79798412323</v>
+        <v>273.6968429088593</v>
       </c>
       <c r="V31" t="inlineStr">
         <is>
@@ -14913,7 +14913,7 @@
         <v>73</v>
       </c>
       <c r="F32" t="n">
-        <v>0.002009153366088867</v>
+        <v>0.001825571060180664</v>
       </c>
       <c r="G32" t="n">
         <v>62</v>
@@ -14925,7 +14925,7 @@
         <v>62</v>
       </c>
       <c r="J32" t="n">
-        <v>14.49254488945007</v>
+        <v>11.36831879615784</v>
       </c>
       <c r="K32" t="n">
         <v>129</v>
@@ -14957,10 +14957,10 @@
         <v>54</v>
       </c>
       <c r="T32" t="n">
-        <v>246.7825529575348</v>
+        <v>197.9426019191742</v>
       </c>
       <c r="U32" t="n">
-        <v>261.277107000351</v>
+        <v>209.3127462863922</v>
       </c>
       <c r="V32" t="inlineStr">
         <is>
@@ -15003,7 +15003,7 @@
         <v>82</v>
       </c>
       <c r="F33" t="n">
-        <v>0.003693103790283203</v>
+        <v>0.001624822616577148</v>
       </c>
       <c r="G33" t="n">
         <v>63</v>
@@ -15015,7 +15015,7 @@
         <v>63</v>
       </c>
       <c r="J33" t="n">
-        <v>9.166265249252319</v>
+        <v>8.00422215461731</v>
       </c>
       <c r="K33" t="n">
         <v>96</v>
@@ -15047,10 +15047,10 @@
         <v>50</v>
       </c>
       <c r="T33" t="n">
-        <v>557.2340369224548</v>
+        <v>401.8620684146881</v>
       </c>
       <c r="U33" t="n">
-        <v>566.4039952754974</v>
+        <v>409.867915391922</v>
       </c>
       <c r="V33" t="inlineStr">
         <is>
@@ -15093,7 +15093,7 @@
         <v>80</v>
       </c>
       <c r="F34" t="n">
-        <v>0.002782821655273438</v>
+        <v>0.001569271087646484</v>
       </c>
       <c r="G34" t="n">
         <v>65</v>
@@ -15105,7 +15105,7 @@
         <v>65</v>
       </c>
       <c r="J34" t="n">
-        <v>22.07341051101685</v>
+        <v>7.997411251068115</v>
       </c>
       <c r="K34" t="n">
         <v>90</v>
@@ -15137,10 +15137,10 @@
         <v>54</v>
       </c>
       <c r="T34" t="n">
-        <v>444.3418323993683</v>
+        <v>332.7426121234894</v>
       </c>
       <c r="U34" t="n">
-        <v>466.4180257320404</v>
+        <v>340.7415926456451</v>
       </c>
       <c r="V34" t="inlineStr">
         <is>
@@ -15183,7 +15183,7 @@
         <v>77</v>
       </c>
       <c r="F35" t="n">
-        <v>0.003633260726928711</v>
+        <v>0.001561403274536133</v>
       </c>
       <c r="G35" t="n">
         <v>59</v>
@@ -15195,7 +15195,7 @@
         <v>59</v>
       </c>
       <c r="J35" t="n">
-        <v>21.13004469871521</v>
+        <v>10.16327142715454</v>
       </c>
       <c r="K35" t="n">
         <v>117</v>
@@ -15227,10 +15227,10 @@
         <v>52</v>
       </c>
       <c r="T35" t="n">
-        <v>434.9264521598816</v>
+        <v>320.6028409004211</v>
       </c>
       <c r="U35" t="n">
-        <v>456.0601301193237</v>
+        <v>330.7676737308502</v>
       </c>
       <c r="V35" t="inlineStr">
         <is>
@@ -15273,7 +15273,7 @@
         <v>82</v>
       </c>
       <c r="F36" t="n">
-        <v>0.002793073654174805</v>
+        <v>0.001505851745605469</v>
       </c>
       <c r="G36" t="n">
         <v>64</v>
@@ -15285,7 +15285,7 @@
         <v>64</v>
       </c>
       <c r="J36" t="n">
-        <v>23.37221336364746</v>
+        <v>9.628232955932617</v>
       </c>
       <c r="K36" t="n">
         <v>116</v>
@@ -15317,10 +15317,10 @@
         <v>50</v>
       </c>
       <c r="T36" t="n">
-        <v>600.1794877052307</v>
+        <v>562.4092059135437</v>
       </c>
       <c r="U36" t="n">
-        <v>623.5544941425323</v>
+        <v>572.0389447212219</v>
       </c>
       <c r="V36" t="inlineStr">
         <is>
@@ -15331,11 +15331,11 @@
         <v>1</v>
       </c>
       <c r="X36" t="n">
-        <v>1475</v>
+        <v>1950</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>t_lim</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -15363,7 +15363,7 @@
         <v>79</v>
       </c>
       <c r="F37" t="n">
-        <v>0.002959012985229492</v>
+        <v>0.003458023071289062</v>
       </c>
       <c r="G37" t="n">
         <v>70</v>
@@ -15375,7 +15375,7 @@
         <v>70</v>
       </c>
       <c r="J37" t="n">
-        <v>5.072072505950928</v>
+        <v>3.832224607467651</v>
       </c>
       <c r="K37" t="n">
         <v>47</v>
@@ -15389,28 +15389,28 @@
         <v>745</v>
       </c>
       <c r="N37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="Q37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T37" t="n">
-        <v>600.1944839954376</v>
+        <v>600.2599928379059</v>
       </c>
       <c r="U37" t="n">
-        <v>605.2695155143738</v>
+        <v>604.0956754684448</v>
       </c>
       <c r="V37" t="inlineStr">
         <is>
@@ -15421,7 +15421,7 @@
         <v>1</v>
       </c>
       <c r="X37" t="n">
-        <v>1530</v>
+        <v>1896</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
@@ -15453,7 +15453,7 @@
         <v>82</v>
       </c>
       <c r="F38" t="n">
-        <v>0.001918554306030273</v>
+        <v>0.001659870147705078</v>
       </c>
       <c r="G38" t="n">
         <v>66</v>
@@ -15465,7 +15465,7 @@
         <v>66</v>
       </c>
       <c r="J38" t="n">
-        <v>7.302220821380615</v>
+        <v>6.053902149200439</v>
       </c>
       <c r="K38" t="n">
         <v>80</v>
@@ -15497,10 +15497,10 @@
         <v>56</v>
       </c>
       <c r="T38" t="n">
-        <v>281.5732188224792</v>
+        <v>272.5439267158508</v>
       </c>
       <c r="U38" t="n">
-        <v>288.8773581981659</v>
+        <v>278.599488735199</v>
       </c>
       <c r="V38" t="inlineStr">
         <is>
@@ -15543,7 +15543,7 @@
         <v>79</v>
       </c>
       <c r="F39" t="n">
-        <v>0.003217935562133789</v>
+        <v>0.003334760665893555</v>
       </c>
       <c r="G39" t="n">
         <v>64</v>
@@ -15555,7 +15555,7 @@
         <v>64</v>
       </c>
       <c r="J39" t="n">
-        <v>17.09362268447876</v>
+        <v>11.16648006439209</v>
       </c>
       <c r="K39" t="n">
         <v>122</v>
@@ -15587,10 +15587,10 @@
         <v>48</v>
       </c>
       <c r="T39" t="n">
-        <v>406.681713104248</v>
+        <v>444.3670554161072</v>
       </c>
       <c r="U39" t="n">
-        <v>423.7785537242889</v>
+        <v>455.5368702411652</v>
       </c>
       <c r="V39" t="inlineStr">
         <is>
@@ -15633,7 +15633,7 @@
         <v>82</v>
       </c>
       <c r="F40" t="n">
-        <v>0.001583576202392578</v>
+        <v>0.001550912857055664</v>
       </c>
       <c r="G40" t="n">
         <v>63</v>
@@ -15645,7 +15645,7 @@
         <v>63</v>
       </c>
       <c r="J40" t="n">
-        <v>10.29624533653259</v>
+        <v>9.921366453170776</v>
       </c>
       <c r="K40" t="n">
         <v>116</v>
@@ -15677,10 +15677,10 @@
         <v>51</v>
       </c>
       <c r="T40" t="n">
-        <v>600.2177696228027</v>
+        <v>600.0046575069427</v>
       </c>
       <c r="U40" t="n">
-        <v>610.5155985355377</v>
+        <v>609.9275748729706</v>
       </c>
       <c r="V40" t="inlineStr">
         <is>
@@ -15691,7 +15691,7 @@
         <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>1706</v>
+        <v>1914</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -15723,7 +15723,7 @@
         <v>79</v>
       </c>
       <c r="F41" t="n">
-        <v>0.006183862686157227</v>
+        <v>0.002007722854614258</v>
       </c>
       <c r="G41" t="n">
         <v>65</v>
@@ -15735,7 +15735,7 @@
         <v>65</v>
       </c>
       <c r="J41" t="n">
-        <v>5.202920913696289</v>
+        <v>4.525194644927979</v>
       </c>
       <c r="K41" t="n">
         <v>55</v>
@@ -15767,10 +15767,10 @@
         <v>50</v>
       </c>
       <c r="T41" t="n">
-        <v>400.3603541851044</v>
+        <v>446.5507719516754</v>
       </c>
       <c r="U41" t="n">
-        <v>405.5694589614868</v>
+        <v>451.077974319458</v>
       </c>
       <c r="V41" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         <v>10</v>
       </c>
       <c r="L2" t="n">
-        <v>2.564436674118042</v>
+        <v>2.652289390563965</v>
       </c>
       <c r="M2" t="n">
         <v>579</v>
@@ -16005,7 +16005,7 @@
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>2.71745777130127</v>
+        <v>3.514975547790527</v>
       </c>
       <c r="M3" t="n">
         <v>644</v>
@@ -16063,7 +16063,7 @@
         <v>10</v>
       </c>
       <c r="L4" t="n">
-        <v>8.255967140197754</v>
+        <v>4.19107723236084</v>
       </c>
       <c r="M4" t="n">
         <v>788</v>
@@ -16121,7 +16121,7 @@
         <v>10</v>
       </c>
       <c r="L5" t="n">
-        <v>2.769766569137573</v>
+        <v>3.228170871734619</v>
       </c>
       <c r="M5" t="n">
         <v>500</v>
@@ -16179,7 +16179,7 @@
         <v>10</v>
       </c>
       <c r="L6" t="n">
-        <v>3.657449245452881</v>
+        <v>3.953996658325195</v>
       </c>
       <c r="M6" t="n">
         <v>560</v>
@@ -16237,7 +16237,7 @@
         <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>2.199610233306885</v>
+        <v>8.113522291183472</v>
       </c>
       <c r="M7" t="n">
         <v>500</v>
@@ -16295,7 +16295,7 @@
         <v>10</v>
       </c>
       <c r="L8" t="n">
-        <v>2.359295606613159</v>
+        <v>2.572837829589844</v>
       </c>
       <c r="M8" t="n">
         <v>500</v>
@@ -16353,7 +16353,7 @@
         <v>10</v>
       </c>
       <c r="L9" t="n">
-        <v>3.043267726898193</v>
+        <v>4.035722970962524</v>
       </c>
       <c r="M9" t="n">
         <v>500</v>
@@ -16411,7 +16411,7 @@
         <v>10</v>
       </c>
       <c r="L10" t="n">
-        <v>2.620037317276001</v>
+        <v>2.831363439559937</v>
       </c>
       <c r="M10" t="n">
         <v>521</v>
@@ -16469,7 +16469,7 @@
         <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>2.135944366455078</v>
+        <v>2.233396768569946</v>
       </c>
       <c r="M11" t="n">
         <v>524</v>
@@ -16527,7 +16527,7 @@
         <v>18</v>
       </c>
       <c r="L12" t="n">
-        <v>7.197542905807495</v>
+        <v>8.463103532791138</v>
       </c>
       <c r="M12" t="n">
         <v>558</v>
@@ -16585,7 +16585,7 @@
         <v>18</v>
       </c>
       <c r="L13" t="n">
-        <v>4.722747564315796</v>
+        <v>5.842691659927368</v>
       </c>
       <c r="M13" t="n">
         <v>506</v>
@@ -16643,7 +16643,7 @@
         <v>16</v>
       </c>
       <c r="L14" t="n">
-        <v>7.404346704483032</v>
+        <v>8.529135704040527</v>
       </c>
       <c r="M14" t="n">
         <v>787</v>
@@ -16701,7 +16701,7 @@
         <v>16</v>
       </c>
       <c r="L15" t="n">
-        <v>4.710891485214233</v>
+        <v>5.819690942764282</v>
       </c>
       <c r="M15" t="n">
         <v>500</v>
@@ -16759,7 +16759,7 @@
         <v>17</v>
       </c>
       <c r="L16" t="n">
-        <v>11.27451801300049</v>
+        <v>12.38631439208984</v>
       </c>
       <c r="M16" t="n">
         <v>989</v>
@@ -16817,7 +16817,7 @@
         <v>18</v>
       </c>
       <c r="L17" t="n">
-        <v>6.062460660934448</v>
+        <v>7.169698715209961</v>
       </c>
       <c r="M17" t="n">
         <v>500</v>
@@ -16875,7 +16875,7 @@
         <v>17</v>
       </c>
       <c r="L18" t="n">
-        <v>5.887769937515259</v>
+        <v>7.005539655685425</v>
       </c>
       <c r="M18" t="n">
         <v>570</v>
@@ -16933,7 +16933,7 @@
         <v>18</v>
       </c>
       <c r="L19" t="n">
-        <v>6.479783535003662</v>
+        <v>7.740480661392212</v>
       </c>
       <c r="M19" t="n">
         <v>602</v>
@@ -16991,7 +16991,7 @@
         <v>17</v>
       </c>
       <c r="L20" t="n">
-        <v>9.089521169662476</v>
+        <v>10.49940276145935</v>
       </c>
       <c r="M20" t="n">
         <v>905</v>
@@ -17049,7 +17049,7 @@
         <v>18</v>
       </c>
       <c r="L21" t="n">
-        <v>4.228868246078491</v>
+        <v>5.332628011703491</v>
       </c>
       <c r="M21" t="n">
         <v>500</v>
@@ -17107,7 +17107,7 @@
         <v>41</v>
       </c>
       <c r="L22" t="n">
-        <v>488.5111601352692</v>
+        <v>337.8674705028534</v>
       </c>
       <c r="M22" t="n">
         <v>1701</v>
@@ -17165,7 +17165,7 @@
         <v>46</v>
       </c>
       <c r="L23" t="n">
-        <v>134.8803567886353</v>
+        <v>106.4561235904694</v>
       </c>
       <c r="M23" t="n">
         <v>500</v>
@@ -17223,7 +17223,7 @@
         <v>39</v>
       </c>
       <c r="L24" t="n">
-        <v>393.8975789546967</v>
+        <v>361.5050694942474</v>
       </c>
       <c r="M24" t="n">
         <v>1875</v>
@@ -17281,7 +17281,7 @@
         <v>39</v>
       </c>
       <c r="L25" t="n">
-        <v>174.9462289810181</v>
+        <v>168.392587184906</v>
       </c>
       <c r="M25" t="n">
         <v>816</v>
@@ -17339,7 +17339,7 @@
         <v>41</v>
       </c>
       <c r="L26" t="n">
-        <v>273.1687104701996</v>
+        <v>246.4103243350983</v>
       </c>
       <c r="M26" t="n">
         <v>1300</v>
@@ -17397,7 +17397,7 @@
         <v>39</v>
       </c>
       <c r="L27" t="n">
-        <v>321.7855217456818</v>
+        <v>290.6666617393494</v>
       </c>
       <c r="M27" t="n">
         <v>1393</v>
@@ -17455,7 +17455,7 @@
         <v>43</v>
       </c>
       <c r="L28" t="n">
-        <v>102.5393631458282</v>
+        <v>98.49638175964355</v>
       </c>
       <c r="M28" t="n">
         <v>513</v>
@@ -17513,7 +17513,7 @@
         <v>41</v>
       </c>
       <c r="L29" t="n">
-        <v>375.0543942451477</v>
+        <v>341.0409514904022</v>
       </c>
       <c r="M29" t="n">
         <v>1550</v>
@@ -17571,7 +17571,7 @@
         <v>38</v>
       </c>
       <c r="L30" t="n">
-        <v>515.514933347702</v>
+        <v>418.7113404273987</v>
       </c>
       <c r="M30" t="n">
         <v>2000</v>
@@ -17629,7 +17629,7 @@
         <v>40</v>
       </c>
       <c r="L31" t="n">
-        <v>307.8504438400269</v>
+        <v>269.7169692516327</v>
       </c>
       <c r="M31" t="n">
         <v>1471</v>
@@ -17687,7 +17687,7 @@
         <v>54</v>
       </c>
       <c r="L32" t="n">
-        <v>246.7825529575348</v>
+        <v>197.9426019191742</v>
       </c>
       <c r="M32" t="n">
         <v>611</v>
@@ -17745,7 +17745,7 @@
         <v>50</v>
       </c>
       <c r="L33" t="n">
-        <v>557.2340369224548</v>
+        <v>401.8620684146881</v>
       </c>
       <c r="M33" t="n">
         <v>1399</v>
@@ -17803,7 +17803,7 @@
         <v>54</v>
       </c>
       <c r="L34" t="n">
-        <v>444.3418323993683</v>
+        <v>332.7426121234894</v>
       </c>
       <c r="M34" t="n">
         <v>1029</v>
@@ -17861,7 +17861,7 @@
         <v>52</v>
       </c>
       <c r="L35" t="n">
-        <v>434.9264521598816</v>
+        <v>320.6028409004211</v>
       </c>
       <c r="M35" t="n">
         <v>982</v>
@@ -17919,14 +17919,14 @@
         <v>50</v>
       </c>
       <c r="L36" t="n">
-        <v>600.1794877052307</v>
+        <v>562.4092059135437</v>
       </c>
       <c r="M36" t="n">
-        <v>1475</v>
+        <v>1950</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>t_lim</t>
+          <t>no_imp_lim</t>
         </is>
       </c>
       <c r="O36" t="b">
@@ -17968,19 +17968,19 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L37" t="n">
-        <v>600.1944839954376</v>
+        <v>600.2599928379059</v>
       </c>
       <c r="M37" t="n">
-        <v>1530</v>
+        <v>1896</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -18035,7 +18035,7 @@
         <v>56</v>
       </c>
       <c r="L38" t="n">
-        <v>281.5732188224792</v>
+        <v>272.5439267158508</v>
       </c>
       <c r="M38" t="n">
         <v>750</v>
@@ -18093,7 +18093,7 @@
         <v>48</v>
       </c>
       <c r="L39" t="n">
-        <v>406.681713104248</v>
+        <v>444.3670554161072</v>
       </c>
       <c r="M39" t="n">
         <v>1330</v>
@@ -18151,10 +18151,10 @@
         <v>51</v>
       </c>
       <c r="L40" t="n">
-        <v>600.2177696228027</v>
+        <v>600.0046575069427</v>
       </c>
       <c r="M40" t="n">
-        <v>1706</v>
+        <v>1914</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -18209,7 +18209,7 @@
         <v>50</v>
       </c>
       <c r="L41" t="n">
-        <v>400.3603541851044</v>
+        <v>446.5507719516754</v>
       </c>
       <c r="M41" t="n">
         <v>1350</v>

</xml_diff>